<commit_message>
Write down model iteratioons and create new sheet for dual work
Create a sheet for Razvans models so that there are no conflicts
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\fae2-nlpr-group-group-12-1\deliverables\Task 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C892E4-6516-4F21-A5A5-E88A731E73EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6250D80D-5FA9-4782-BE90-C5C06FDF1D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
+    <workbookView xWindow="-15" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Model Iteration Log" sheetId="1" r:id="rId1"/>
+    <sheet name="Model Iteration Log Filip" sheetId="1" r:id="rId1"/>
+    <sheet name="Model Iteration Log Razvan" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="67">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -218,16 +219,43 @@
     <t>0.274</t>
   </si>
   <si>
-    <t>0.256</t>
-  </si>
-  <si>
-    <t>0.225</t>
-  </si>
-  <si>
-    <t>0.205</t>
-  </si>
-  <si>
     <t>Overall best performing among these models</t>
+  </si>
+  <si>
+    <t>0.248</t>
+  </si>
+  <si>
+    <t>0.220</t>
+  </si>
+  <si>
+    <t>0.219</t>
+  </si>
+  <si>
+    <t>ax_iter=3000, penalty='elasticnet', random_state=42, solver='saga', l1_ratio=0.5</t>
+  </si>
+  <si>
+    <t>0.252</t>
+  </si>
+  <si>
+    <t>var_smoothing=2</t>
+  </si>
+  <si>
+    <t>0.287</t>
+  </si>
+  <si>
+    <t>0.233</t>
+  </si>
+  <si>
+    <t>0.234</t>
+  </si>
+  <si>
+    <t>0.260</t>
+  </si>
+  <si>
+    <t>0.202</t>
+  </si>
+  <si>
+    <t>0.211</t>
   </si>
 </sst>
 </file>
@@ -1266,7 +1294,7 @@
       </c>
       <c r="O12" s="10"/>
       <c r="P12" s="10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="Q12" s="10"/>
       <c r="R12" s="10"/>
@@ -1304,13 +1332,13 @@
         <v>42</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="N13" s="10" t="s">
         <v>56</v>
@@ -1355,11 +1383,21 @@
       <c r="I14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
+      <c r="J14" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>57</v>
+      </c>
       <c r="O14" s="10"/>
       <c r="P14" s="10"/>
       <c r="Q14" s="10"/>
@@ -1371,18 +1409,40 @@
       <c r="B15" s="9">
         <v>5</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
+      <c r="C15" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>46</v>
+      </c>
       <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
+      <c r="J15" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>63</v>
+      </c>
       <c r="O15" s="10"/>
       <c r="P15" s="10"/>
       <c r="Q15" s="10"/>
@@ -1394,18 +1454,38 @@
       <c r="B16" s="9">
         <v>6</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="C16" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>32</v>
+      </c>
       <c r="H16" s="10"/>
       <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
+      <c r="J16" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="L16" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="M16" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>66</v>
+      </c>
       <c r="O16" s="10"/>
       <c r="P16" s="10"/>
       <c r="Q16" s="10"/>
@@ -2212,4 +2292,1373 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F6E3FC4-92B9-4B14-9A38-1F80DD1D104A}">
+  <dimension ref="B2:U51"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="6.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20" style="1" customWidth="1"/>
+    <col min="6" max="6" width="36" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="32" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5703125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5703125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.42578125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="33.140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5703125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="31.42578125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.28515625" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+      <c r="B2" s="2"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+      <c r="B3" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="28"/>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="29"/>
+      <c r="U3" s="5"/>
+    </row>
+    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="6"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="8"/>
+    </row>
+    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="6"/>
+      <c r="C5" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="19"/>
+    </row>
+    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="6"/>
+      <c r="C6" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="19"/>
+    </row>
+    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="6"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="19"/>
+    </row>
+    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="6"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="18"/>
+      <c r="T8" s="19"/>
+    </row>
+    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="16"/>
+      <c r="C9" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="30"/>
+      <c r="E9" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="K9" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="31"/>
+      <c r="P9" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q9" s="30"/>
+      <c r="R9" s="30"/>
+      <c r="S9" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="T9" s="23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="N10" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="O10" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="P10" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q10" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="R10" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="S10" s="25"/>
+      <c r="T10" s="26"/>
+    </row>
+    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="9">
+        <v>1</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L11" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="R11" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="S11" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="T11" s="11"/>
+    </row>
+    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="9">
+        <v>2</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
+      <c r="S12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="T12" s="11"/>
+    </row>
+    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="9">
+        <v>3</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q13" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="R13" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="S13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="T13" s="11"/>
+    </row>
+    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="9">
+        <v>4</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="11"/>
+    </row>
+    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="9">
+        <v>5</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="11"/>
+    </row>
+    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="9">
+        <v>6</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="L16" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="M16" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="10"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="11"/>
+    </row>
+    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="9">
+        <v>7</v>
+      </c>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="11"/>
+    </row>
+    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="9">
+        <v>8</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="11"/>
+    </row>
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="9">
+        <v>9</v>
+      </c>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="11"/>
+    </row>
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="9">
+        <v>10</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="11"/>
+    </row>
+    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="9">
+        <v>11</v>
+      </c>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="11"/>
+    </row>
+    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="9">
+        <v>12</v>
+      </c>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="10"/>
+      <c r="S22" s="10"/>
+      <c r="T22" s="11"/>
+    </row>
+    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="9">
+        <v>13</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10"/>
+      <c r="T23" s="11"/>
+    </row>
+    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="9">
+        <v>14</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="10"/>
+      <c r="S24" s="10"/>
+      <c r="T24" s="11"/>
+    </row>
+    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="9">
+        <v>15</v>
+      </c>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="10"/>
+      <c r="S25" s="10"/>
+      <c r="T25" s="11"/>
+    </row>
+    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="9">
+        <v>16</v>
+      </c>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10"/>
+      <c r="T26" s="11"/>
+    </row>
+    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="9">
+        <v>17</v>
+      </c>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="10"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="10"/>
+      <c r="S27" s="10"/>
+      <c r="T27" s="11"/>
+    </row>
+    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="9">
+        <v>18</v>
+      </c>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="10"/>
+      <c r="S28" s="10"/>
+      <c r="T28" s="11"/>
+    </row>
+    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="9">
+        <v>19</v>
+      </c>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+      <c r="T29" s="11"/>
+    </row>
+    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="9">
+        <v>20</v>
+      </c>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="11"/>
+    </row>
+    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="9">
+        <v>21</v>
+      </c>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="10"/>
+      <c r="S31" s="10"/>
+      <c r="T31" s="11"/>
+    </row>
+    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="9">
+        <v>22</v>
+      </c>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10"/>
+      <c r="N32" s="10"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="10"/>
+      <c r="S32" s="10"/>
+      <c r="T32" s="11"/>
+    </row>
+    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="9">
+        <v>23</v>
+      </c>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="10"/>
+      <c r="S33" s="10"/>
+      <c r="T33" s="11"/>
+    </row>
+    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="9">
+        <v>24</v>
+      </c>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="10"/>
+      <c r="S34" s="10"/>
+      <c r="T34" s="11"/>
+    </row>
+    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="9">
+        <v>25</v>
+      </c>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="10"/>
+      <c r="M35" s="10"/>
+      <c r="N35" s="10"/>
+      <c r="O35" s="10"/>
+      <c r="P35" s="10"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="10"/>
+      <c r="S35" s="10"/>
+      <c r="T35" s="11"/>
+    </row>
+    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="9">
+        <v>26</v>
+      </c>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="10"/>
+      <c r="N36" s="10"/>
+      <c r="O36" s="10"/>
+      <c r="P36" s="10"/>
+      <c r="Q36" s="10"/>
+      <c r="R36" s="10"/>
+      <c r="S36" s="10"/>
+      <c r="T36" s="11"/>
+    </row>
+    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="9">
+        <v>27</v>
+      </c>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
+      <c r="Q37" s="10"/>
+      <c r="R37" s="10"/>
+      <c r="S37" s="10"/>
+      <c r="T37" s="11"/>
+    </row>
+    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="9">
+        <v>28</v>
+      </c>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
+      <c r="N38" s="10"/>
+      <c r="O38" s="10"/>
+      <c r="P38" s="10"/>
+      <c r="Q38" s="10"/>
+      <c r="R38" s="10"/>
+      <c r="S38" s="10"/>
+      <c r="T38" s="11"/>
+    </row>
+    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="9">
+        <v>29</v>
+      </c>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="10"/>
+      <c r="O39" s="10"/>
+      <c r="P39" s="10"/>
+      <c r="Q39" s="10"/>
+      <c r="R39" s="10"/>
+      <c r="S39" s="10"/>
+      <c r="T39" s="11"/>
+    </row>
+    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="9">
+        <v>30</v>
+      </c>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+      <c r="O40" s="10"/>
+      <c r="P40" s="10"/>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="10"/>
+      <c r="S40" s="10"/>
+      <c r="T40" s="11"/>
+    </row>
+    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="9">
+        <v>31</v>
+      </c>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+      <c r="M41" s="10"/>
+      <c r="N41" s="10"/>
+      <c r="O41" s="10"/>
+      <c r="P41" s="10"/>
+      <c r="Q41" s="10"/>
+      <c r="R41" s="10"/>
+      <c r="S41" s="10"/>
+      <c r="T41" s="11"/>
+    </row>
+    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="9">
+        <v>32</v>
+      </c>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10"/>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+      <c r="M42" s="10"/>
+      <c r="N42" s="10"/>
+      <c r="O42" s="10"/>
+      <c r="P42" s="10"/>
+      <c r="Q42" s="10"/>
+      <c r="R42" s="10"/>
+      <c r="S42" s="10"/>
+      <c r="T42" s="11"/>
+    </row>
+    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="9">
+        <v>33</v>
+      </c>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
+      <c r="N43" s="10"/>
+      <c r="O43" s="10"/>
+      <c r="P43" s="10"/>
+      <c r="Q43" s="10"/>
+      <c r="R43" s="10"/>
+      <c r="S43" s="10"/>
+      <c r="T43" s="11"/>
+    </row>
+    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="9">
+        <v>34</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="10"/>
+      <c r="N44" s="10"/>
+      <c r="O44" s="10"/>
+      <c r="P44" s="10"/>
+      <c r="Q44" s="10"/>
+      <c r="R44" s="10"/>
+      <c r="S44" s="10"/>
+      <c r="T44" s="11"/>
+    </row>
+    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="9">
+        <v>35</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
+      <c r="J45" s="10"/>
+      <c r="K45" s="10"/>
+      <c r="L45" s="10"/>
+      <c r="M45" s="10"/>
+      <c r="N45" s="10"/>
+      <c r="O45" s="10"/>
+      <c r="P45" s="10"/>
+      <c r="Q45" s="10"/>
+      <c r="R45" s="10"/>
+      <c r="S45" s="10"/>
+      <c r="T45" s="11"/>
+    </row>
+    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="9">
+        <v>36</v>
+      </c>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
+      <c r="J46" s="10"/>
+      <c r="K46" s="10"/>
+      <c r="L46" s="10"/>
+      <c r="M46" s="10"/>
+      <c r="N46" s="10"/>
+      <c r="O46" s="10"/>
+      <c r="P46" s="10"/>
+      <c r="Q46" s="10"/>
+      <c r="R46" s="10"/>
+      <c r="S46" s="10"/>
+      <c r="T46" s="11"/>
+    </row>
+    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="9">
+        <v>37</v>
+      </c>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="10"/>
+      <c r="K47" s="10"/>
+      <c r="L47" s="10"/>
+      <c r="M47" s="10"/>
+      <c r="N47" s="10"/>
+      <c r="O47" s="10"/>
+      <c r="P47" s="10"/>
+      <c r="Q47" s="10"/>
+      <c r="R47" s="10"/>
+      <c r="S47" s="10"/>
+      <c r="T47" s="11"/>
+    </row>
+    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="9">
+        <v>38</v>
+      </c>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10"/>
+      <c r="J48" s="10"/>
+      <c r="K48" s="10"/>
+      <c r="L48" s="10"/>
+      <c r="M48" s="10"/>
+      <c r="N48" s="10"/>
+      <c r="O48" s="10"/>
+      <c r="P48" s="10"/>
+      <c r="Q48" s="10"/>
+      <c r="R48" s="10"/>
+      <c r="S48" s="10"/>
+      <c r="T48" s="11"/>
+    </row>
+    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="9">
+        <v>39</v>
+      </c>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
+      <c r="L49" s="10"/>
+      <c r="M49" s="10"/>
+      <c r="N49" s="10"/>
+      <c r="O49" s="10"/>
+      <c r="P49" s="10"/>
+      <c r="Q49" s="10"/>
+      <c r="R49" s="10"/>
+      <c r="S49" s="10"/>
+      <c r="T49" s="11"/>
+    </row>
+    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="12">
+        <v>40</v>
+      </c>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="13"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="13"/>
+      <c r="K50" s="13"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="13"/>
+      <c r="N50" s="13"/>
+      <c r="O50" s="13"/>
+      <c r="P50" s="13"/>
+      <c r="Q50" s="13"/>
+      <c r="R50" s="13"/>
+      <c r="S50" s="13"/>
+      <c r="T50" s="14"/>
+    </row>
+    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C51" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:I9"/>
+    <mergeCell ref="K9:O9"/>
+    <mergeCell ref="P9:R9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Iterate models, write them down into the iteration log
Performed few more iteration of sklearn models to try and increase the scores. Noted down these scores in the log
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6250D80D-5FA9-4782-BE90-C5C06FDF1D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9FE50D-D74E-4C3F-9993-3836926AD336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="71">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -256,6 +256,18 @@
   </si>
   <si>
     <t>0.211</t>
+  </si>
+  <si>
+    <t>penalty='l2', loss='squared_hinge', C=2000.0, multi_class='ovr', fit_intercept=True, random_state=42, dual=True, max_iter=30000</t>
+  </si>
+  <si>
+    <t>0.262</t>
+  </si>
+  <si>
+    <t>0.206</t>
+  </si>
+  <si>
+    <t>0.214</t>
   </si>
 </sst>
 </file>
@@ -2588,9 +2600,7 @@
       <c r="H11" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I11" s="10" t="s">
-        <v>47</v>
-      </c>
+      <c r="I11" s="10"/>
       <c r="J11" s="10" t="s">
         <v>34</v>
       </c>
@@ -2643,9 +2653,7 @@
       <c r="H12" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I12" s="10" t="s">
-        <v>47</v>
-      </c>
+      <c r="I12" s="10"/>
       <c r="J12" s="10" t="s">
         <v>40</v>
       </c>
@@ -2694,9 +2702,7 @@
       <c r="H13" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I13" s="10" t="s">
-        <v>47</v>
-      </c>
+      <c r="I13" s="10"/>
       <c r="J13" s="10" t="s">
         <v>42</v>
       </c>
@@ -2749,9 +2755,7 @@
       <c r="H14" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="I14" s="10" t="s">
-        <v>47</v>
-      </c>
+      <c r="I14" s="10"/>
       <c r="J14" s="10" t="s">
         <v>58</v>
       </c>
@@ -2838,22 +2842,24 @@
       <c r="G16" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="10"/>
+      <c r="H16" s="10" t="s">
+        <v>46</v>
+      </c>
       <c r="I16" s="10"/>
       <c r="J16" s="10" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="O16" s="10"/>
       <c r="P16" s="10"/>

</xml_diff>

<commit_message>
Update RNN and LSTM models
I updated the RNN and LSTM models  and logged them in the model iteration file
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\git-school\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6250D80D-5FA9-4782-BE90-C5C06FDF1D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F9D2EA-9C7D-4EFD-B1BD-49E93B52BFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
   <sheets>
     <sheet name="Model Iteration Log Filip" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="75">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -257,12 +257,36 @@
   <si>
     <t>0.211</t>
   </si>
+  <si>
+    <t>SimpleRNN</t>
+  </si>
+  <si>
+    <t>keras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">features.py (baseline) + tf.keras.preprocessing.text.Tokenizer and tf.keras.preprocessing.sequence.pad_sequences </t>
+  </si>
+  <si>
+    <t>Sentence_Tok'</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>lr=1e-4, kernel_regularizer="l2" for the dense layers, batch_size=64</t>
+  </si>
+  <si>
+    <t>LSTM</t>
+  </si>
+  <si>
+    <t>lr=5e-3, kernel_regularizer="l2" for the dense layers, batch_size=64</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,6 +355,12 @@
       <name val="Aptos Display"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -494,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -571,6 +601,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -928,31 +961,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10A5CD43-FACF-4F92-BDE3-5E7B47D72998}">
   <dimension ref="B2:U51"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="6.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="6.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="36" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="32" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="33.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="31.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="20.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="33.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.33203125" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -974,31 +1007,31 @@
       <c r="T2" s="4"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="2:21" ht="24" x14ac:dyDescent="0.4">
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B3" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="28"/>
-      <c r="S3" s="28"/>
-      <c r="T3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="30"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -1019,18 +1052,18 @@
       <c r="S4" s="7"/>
       <c r="T4" s="8"/>
     </row>
-    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6"/>
       <c r="C5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -1042,18 +1075,18 @@
       <c r="S5" s="18"/>
       <c r="T5" s="19"/>
     </row>
-    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
       <c r="C6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
@@ -1065,7 +1098,7 @@
       <c r="S6" s="18"/>
       <c r="T6" s="19"/>
     </row>
-    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6"/>
       <c r="C7" s="18"/>
       <c r="D7" s="20"/>
@@ -1086,7 +1119,7 @@
       <c r="S7" s="18"/>
       <c r="T7" s="19"/>
     </row>
-    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6"/>
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
@@ -1107,34 +1140,34 @@
       <c r="S8" s="18"/>
       <c r="T8" s="19"/>
     </row>
-    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="16"/>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="31" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
       <c r="J9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="31" t="s">
+      <c r="K9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="31"/>
-      <c r="P9" s="30" t="s">
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="31"/>
       <c r="S9" s="22" t="s">
         <v>24</v>
       </c>
@@ -1142,7 +1175,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>7</v>
       </c>
@@ -1197,7 +1230,7 @@
       <c r="S10" s="25"/>
       <c r="T10" s="26"/>
     </row>
-    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="9">
         <v>1</v>
       </c>
@@ -1252,7 +1285,7 @@
       </c>
       <c r="T11" s="11"/>
     </row>
-    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>2</v>
       </c>
@@ -1303,7 +1336,7 @@
       </c>
       <c r="T12" s="11"/>
     </row>
-    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
         <v>3</v>
       </c>
@@ -1358,7 +1391,7 @@
       </c>
       <c r="T13" s="11"/>
     </row>
-    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="9">
         <v>4</v>
       </c>
@@ -1405,7 +1438,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="11"/>
     </row>
-    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="9">
         <v>5</v>
       </c>
@@ -1450,7 +1483,7 @@
       <c r="S15" s="10"/>
       <c r="T15" s="11"/>
     </row>
-    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="9">
         <v>6</v>
       </c>
@@ -1493,7 +1526,7 @@
       <c r="S16" s="10"/>
       <c r="T16" s="11"/>
     </row>
-    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="9">
         <v>7</v>
       </c>
@@ -1516,7 +1549,7 @@
       <c r="S17" s="10"/>
       <c r="T17" s="11"/>
     </row>
-    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9">
         <v>8</v>
       </c>
@@ -1539,7 +1572,7 @@
       <c r="S18" s="10"/>
       <c r="T18" s="11"/>
     </row>
-    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>9</v>
       </c>
@@ -1562,7 +1595,7 @@
       <c r="S19" s="10"/>
       <c r="T19" s="11"/>
     </row>
-    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="9">
         <v>10</v>
       </c>
@@ -1585,7 +1618,7 @@
       <c r="S20" s="10"/>
       <c r="T20" s="11"/>
     </row>
-    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9">
         <v>11</v>
       </c>
@@ -1608,7 +1641,7 @@
       <c r="S21" s="10"/>
       <c r="T21" s="11"/>
     </row>
-    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
         <v>12</v>
       </c>
@@ -1631,7 +1664,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="11"/>
     </row>
-    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
@@ -1654,7 +1687,7 @@
       <c r="S23" s="10"/>
       <c r="T23" s="11"/>
     </row>
-    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9">
         <v>14</v>
       </c>
@@ -1677,7 +1710,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="11"/>
     </row>
-    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9">
         <v>15</v>
       </c>
@@ -1700,7 +1733,7 @@
       <c r="S25" s="10"/>
       <c r="T25" s="11"/>
     </row>
-    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
         <v>16</v>
       </c>
@@ -1723,7 +1756,7 @@
       <c r="S26" s="10"/>
       <c r="T26" s="11"/>
     </row>
-    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="9">
         <v>17</v>
       </c>
@@ -1746,7 +1779,7 @@
       <c r="S27" s="10"/>
       <c r="T27" s="11"/>
     </row>
-    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="9">
         <v>18</v>
       </c>
@@ -1769,7 +1802,7 @@
       <c r="S28" s="10"/>
       <c r="T28" s="11"/>
     </row>
-    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="9">
         <v>19</v>
       </c>
@@ -1792,7 +1825,7 @@
       <c r="S29" s="10"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="9">
         <v>20</v>
       </c>
@@ -1815,7 +1848,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="11"/>
     </row>
-    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="9">
         <v>21</v>
       </c>
@@ -1838,7 +1871,7 @@
       <c r="S31" s="10"/>
       <c r="T31" s="11"/>
     </row>
-    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9">
         <v>22</v>
       </c>
@@ -1861,7 +1894,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="11"/>
     </row>
-    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="9">
         <v>23</v>
       </c>
@@ -1884,7 +1917,7 @@
       <c r="S33" s="10"/>
       <c r="T33" s="11"/>
     </row>
-    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="9">
         <v>24</v>
       </c>
@@ -1907,7 +1940,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="11"/>
     </row>
-    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="9">
         <v>25</v>
       </c>
@@ -1930,7 +1963,7 @@
       <c r="S35" s="10"/>
       <c r="T35" s="11"/>
     </row>
-    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9">
         <v>26</v>
       </c>
@@ -1953,7 +1986,7 @@
       <c r="S36" s="10"/>
       <c r="T36" s="11"/>
     </row>
-    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="9">
         <v>27</v>
       </c>
@@ -1976,7 +2009,7 @@
       <c r="S37" s="10"/>
       <c r="T37" s="11"/>
     </row>
-    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="9">
         <v>28</v>
       </c>
@@ -1999,7 +2032,7 @@
       <c r="S38" s="10"/>
       <c r="T38" s="11"/>
     </row>
-    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
         <v>29</v>
       </c>
@@ -2022,7 +2055,7 @@
       <c r="S39" s="10"/>
       <c r="T39" s="11"/>
     </row>
-    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9">
         <v>30</v>
       </c>
@@ -2045,7 +2078,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="11"/>
     </row>
-    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="9">
         <v>31</v>
       </c>
@@ -2068,7 +2101,7 @@
       <c r="S41" s="10"/>
       <c r="T41" s="11"/>
     </row>
-    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="9">
         <v>32</v>
       </c>
@@ -2091,7 +2124,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="11"/>
     </row>
-    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="9">
         <v>33</v>
       </c>
@@ -2114,7 +2147,7 @@
       <c r="S43" s="10"/>
       <c r="T43" s="11"/>
     </row>
-    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="9">
         <v>34</v>
       </c>
@@ -2137,7 +2170,7 @@
       <c r="S44" s="10"/>
       <c r="T44" s="11"/>
     </row>
-    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="9">
         <v>35</v>
       </c>
@@ -2160,7 +2193,7 @@
       <c r="S45" s="10"/>
       <c r="T45" s="11"/>
     </row>
-    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="9">
         <v>36</v>
       </c>
@@ -2183,7 +2216,7 @@
       <c r="S46" s="10"/>
       <c r="T46" s="11"/>
     </row>
-    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="9">
         <v>37</v>
       </c>
@@ -2206,7 +2239,7 @@
       <c r="S47" s="10"/>
       <c r="T47" s="11"/>
     </row>
-    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="9">
         <v>38</v>
       </c>
@@ -2229,7 +2262,7 @@
       <c r="S48" s="10"/>
       <c r="T48" s="11"/>
     </row>
-    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="9">
         <v>39</v>
       </c>
@@ -2252,7 +2285,7 @@
       <c r="S49" s="10"/>
       <c r="T49" s="11"/>
     </row>
-    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12">
         <v>40</v>
       </c>
@@ -2275,7 +2308,7 @@
       <c r="S50" s="13"/>
       <c r="T50" s="14"/>
     </row>
-    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C51" s="15" t="s">
         <v>8</v>
       </c>
@@ -2297,31 +2330,31 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F6E3FC4-92B9-4B14-9A38-1F80DD1D104A}">
   <dimension ref="B2:U51"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="6.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="6.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="36" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="32" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="33.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="31.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="20.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="33.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.33203125" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2343,31 +2376,31 @@
       <c r="T2" s="4"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="2:21" ht="24" x14ac:dyDescent="0.4">
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B3" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="28"/>
-      <c r="S3" s="28"/>
-      <c r="T3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="30"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -2388,18 +2421,18 @@
       <c r="S4" s="7"/>
       <c r="T4" s="8"/>
     </row>
-    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6"/>
       <c r="C5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -2411,18 +2444,18 @@
       <c r="S5" s="18"/>
       <c r="T5" s="19"/>
     </row>
-    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
       <c r="C6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
@@ -2434,7 +2467,7 @@
       <c r="S6" s="18"/>
       <c r="T6" s="19"/>
     </row>
-    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6"/>
       <c r="C7" s="18"/>
       <c r="D7" s="20"/>
@@ -2455,7 +2488,7 @@
       <c r="S7" s="18"/>
       <c r="T7" s="19"/>
     </row>
-    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6"/>
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
@@ -2476,34 +2509,34 @@
       <c r="S8" s="18"/>
       <c r="T8" s="19"/>
     </row>
-    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="16"/>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="31" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
       <c r="J9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="31" t="s">
+      <c r="K9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="31"/>
-      <c r="P9" s="30" t="s">
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="31"/>
       <c r="S9" s="22" t="s">
         <v>24</v>
       </c>
@@ -2511,7 +2544,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>7</v>
       </c>
@@ -2566,7 +2599,7 @@
       <c r="S10" s="25"/>
       <c r="T10" s="26"/>
     </row>
-    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="9">
         <v>1</v>
       </c>
@@ -2594,17 +2627,17 @@
       <c r="J11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="K11" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="L11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="N11" s="10" t="s">
-        <v>50</v>
+      <c r="K11" s="10">
+        <v>0.24399999999999999</v>
+      </c>
+      <c r="L11" s="10">
+        <v>0.224</v>
+      </c>
+      <c r="M11" s="10">
+        <v>0.224</v>
+      </c>
+      <c r="N11" s="10">
+        <v>0.216</v>
       </c>
       <c r="O11" s="10"/>
       <c r="P11" s="10" t="s">
@@ -2621,7 +2654,7 @@
       </c>
       <c r="T11" s="11"/>
     </row>
-    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>2</v>
       </c>
@@ -2649,17 +2682,17 @@
       <c r="J12" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="N12" s="10" t="s">
-        <v>53</v>
+      <c r="K12" s="10">
+        <v>0.29299999999999998</v>
+      </c>
+      <c r="L12" s="10">
+        <v>0.29099999999999998</v>
+      </c>
+      <c r="M12" s="10">
+        <v>0.29299999999999998</v>
+      </c>
+      <c r="N12" s="10">
+        <v>0.27400000000000002</v>
       </c>
       <c r="O12" s="10"/>
       <c r="P12" s="10" t="s">
@@ -2672,7 +2705,7 @@
       </c>
       <c r="T12" s="11"/>
     </row>
-    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
         <v>3</v>
       </c>
@@ -2700,17 +2733,17 @@
       <c r="J13" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="K13" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="L13" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="N13" s="10" t="s">
-        <v>56</v>
+      <c r="K13" s="10">
+        <v>0.252</v>
+      </c>
+      <c r="L13" s="10">
+        <v>0.216</v>
+      </c>
+      <c r="M13" s="10">
+        <v>0.252</v>
+      </c>
+      <c r="N13" s="10">
+        <v>0.22</v>
       </c>
       <c r="O13" s="10"/>
       <c r="P13" s="10" t="s">
@@ -2727,7 +2760,7 @@
       </c>
       <c r="T13" s="11"/>
     </row>
-    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="9">
         <v>4</v>
       </c>
@@ -2755,17 +2788,17 @@
       <c r="J14" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="K14" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="M14" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="N14" s="10" t="s">
-        <v>57</v>
+      <c r="K14" s="10">
+        <v>0.248</v>
+      </c>
+      <c r="L14" s="10">
+        <v>0.22</v>
+      </c>
+      <c r="M14" s="10">
+        <v>0.248</v>
+      </c>
+      <c r="N14" s="10">
+        <v>0.219</v>
       </c>
       <c r="O14" s="10"/>
       <c r="P14" s="10"/>
@@ -2774,7 +2807,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="11"/>
     </row>
-    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="9">
         <v>5</v>
       </c>
@@ -2800,17 +2833,17 @@
       <c r="J15" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="K15" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="L15" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="N15" s="10" t="s">
-        <v>63</v>
+      <c r="K15" s="10">
+        <v>0.28699999999999998</v>
+      </c>
+      <c r="L15" s="10">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="M15" s="10">
+        <v>0.28699999999999998</v>
+      </c>
+      <c r="N15" s="10">
+        <v>0.23400000000000001</v>
       </c>
       <c r="O15" s="10"/>
       <c r="P15" s="10"/>
@@ -2819,7 +2852,7 @@
       <c r="S15" s="10"/>
       <c r="T15" s="11"/>
     </row>
-    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="9">
         <v>6</v>
       </c>
@@ -2843,17 +2876,17 @@
       <c r="J16" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="K16" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="N16" s="10" t="s">
-        <v>66</v>
+      <c r="K16" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="L16" s="10">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="M16" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="N16" s="10">
+        <v>0.21099999999999999</v>
       </c>
       <c r="O16" s="10"/>
       <c r="P16" s="10"/>
@@ -2862,22 +2895,46 @@
       <c r="S16" s="10"/>
       <c r="T16" s="11"/>
     </row>
-    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="9">
         <v>7</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
+      <c r="C17" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="K17" s="10">
+        <v>0.56399999999999995</v>
+      </c>
+      <c r="L17" s="10">
+        <v>0.56499999999999995</v>
+      </c>
+      <c r="M17" s="10">
+        <v>0.56399999999999995</v>
+      </c>
+      <c r="N17" s="10">
+        <v>0.56299999999999994</v>
+      </c>
       <c r="O17" s="10"/>
       <c r="P17" s="10"/>
       <c r="Q17" s="10"/>
@@ -2885,22 +2942,46 @@
       <c r="S17" s="10"/>
       <c r="T17" s="11"/>
     </row>
-    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9">
         <v>8</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
+      <c r="C18" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H18" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="K18" s="10">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="L18" s="10">
+        <v>0.77800000000000002</v>
+      </c>
+      <c r="M18" s="10">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="N18" s="10">
+        <v>0.76700000000000002</v>
+      </c>
       <c r="O18" s="10"/>
       <c r="P18" s="10"/>
       <c r="Q18" s="10"/>
@@ -2908,7 +2989,7 @@
       <c r="S18" s="10"/>
       <c r="T18" s="11"/>
     </row>
-    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>9</v>
       </c>
@@ -2931,7 +3012,7 @@
       <c r="S19" s="10"/>
       <c r="T19" s="11"/>
     </row>
-    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="9">
         <v>10</v>
       </c>
@@ -2954,7 +3035,7 @@
       <c r="S20" s="10"/>
       <c r="T20" s="11"/>
     </row>
-    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9">
         <v>11</v>
       </c>
@@ -2977,7 +3058,7 @@
       <c r="S21" s="10"/>
       <c r="T21" s="11"/>
     </row>
-    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
         <v>12</v>
       </c>
@@ -3000,7 +3081,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="11"/>
     </row>
-    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
@@ -3023,7 +3104,7 @@
       <c r="S23" s="10"/>
       <c r="T23" s="11"/>
     </row>
-    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9">
         <v>14</v>
       </c>
@@ -3046,7 +3127,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="11"/>
     </row>
-    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9">
         <v>15</v>
       </c>
@@ -3069,7 +3150,7 @@
       <c r="S25" s="10"/>
       <c r="T25" s="11"/>
     </row>
-    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
         <v>16</v>
       </c>
@@ -3092,7 +3173,7 @@
       <c r="S26" s="10"/>
       <c r="T26" s="11"/>
     </row>
-    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="9">
         <v>17</v>
       </c>
@@ -3115,7 +3196,7 @@
       <c r="S27" s="10"/>
       <c r="T27" s="11"/>
     </row>
-    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="9">
         <v>18</v>
       </c>
@@ -3138,7 +3219,7 @@
       <c r="S28" s="10"/>
       <c r="T28" s="11"/>
     </row>
-    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="9">
         <v>19</v>
       </c>
@@ -3161,7 +3242,7 @@
       <c r="S29" s="10"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="9">
         <v>20</v>
       </c>
@@ -3184,7 +3265,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="11"/>
     </row>
-    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="9">
         <v>21</v>
       </c>
@@ -3207,7 +3288,7 @@
       <c r="S31" s="10"/>
       <c r="T31" s="11"/>
     </row>
-    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9">
         <v>22</v>
       </c>
@@ -3230,7 +3311,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="11"/>
     </row>
-    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="9">
         <v>23</v>
       </c>
@@ -3253,7 +3334,7 @@
       <c r="S33" s="10"/>
       <c r="T33" s="11"/>
     </row>
-    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="9">
         <v>24</v>
       </c>
@@ -3276,7 +3357,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="11"/>
     </row>
-    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="9">
         <v>25</v>
       </c>
@@ -3299,7 +3380,7 @@
       <c r="S35" s="10"/>
       <c r="T35" s="11"/>
     </row>
-    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9">
         <v>26</v>
       </c>
@@ -3322,7 +3403,7 @@
       <c r="S36" s="10"/>
       <c r="T36" s="11"/>
     </row>
-    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="9">
         <v>27</v>
       </c>
@@ -3345,7 +3426,7 @@
       <c r="S37" s="10"/>
       <c r="T37" s="11"/>
     </row>
-    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="9">
         <v>28</v>
       </c>
@@ -3368,7 +3449,7 @@
       <c r="S38" s="10"/>
       <c r="T38" s="11"/>
     </row>
-    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
         <v>29</v>
       </c>
@@ -3391,7 +3472,7 @@
       <c r="S39" s="10"/>
       <c r="T39" s="11"/>
     </row>
-    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9">
         <v>30</v>
       </c>
@@ -3414,7 +3495,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="11"/>
     </row>
-    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="9">
         <v>31</v>
       </c>
@@ -3437,7 +3518,7 @@
       <c r="S41" s="10"/>
       <c r="T41" s="11"/>
     </row>
-    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="9">
         <v>32</v>
       </c>
@@ -3460,7 +3541,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="11"/>
     </row>
-    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="9">
         <v>33</v>
       </c>
@@ -3483,7 +3564,7 @@
       <c r="S43" s="10"/>
       <c r="T43" s="11"/>
     </row>
-    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="9">
         <v>34</v>
       </c>
@@ -3506,7 +3587,7 @@
       <c r="S44" s="10"/>
       <c r="T44" s="11"/>
     </row>
-    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="9">
         <v>35</v>
       </c>
@@ -3529,7 +3610,7 @@
       <c r="S45" s="10"/>
       <c r="T45" s="11"/>
     </row>
-    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="9">
         <v>36</v>
       </c>
@@ -3552,7 +3633,7 @@
       <c r="S46" s="10"/>
       <c r="T46" s="11"/>
     </row>
-    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="9">
         <v>37</v>
       </c>
@@ -3575,7 +3656,7 @@
       <c r="S47" s="10"/>
       <c r="T47" s="11"/>
     </row>
-    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="9">
         <v>38</v>
       </c>
@@ -3598,7 +3679,7 @@
       <c r="S48" s="10"/>
       <c r="T48" s="11"/>
     </row>
-    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="9">
         <v>39</v>
       </c>
@@ -3621,7 +3702,7 @@
       <c r="S49" s="10"/>
       <c r="T49" s="11"/>
     </row>
-    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12">
         <v>40</v>
       </c>
@@ -3644,7 +3725,7 @@
       <c r="S50" s="13"/>
       <c r="T50" s="14"/>
     </row>
-    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C51" s="15" t="s">
         <v>8</v>
       </c>
@@ -3659,6 +3740,7 @@
     <mergeCell ref="K9:O9"/>
     <mergeCell ref="P9:R9"/>
   </mergeCells>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restored Y2A_model_iteration_log.xlsx from commit 2da9f2d
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\git-school\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9FE50D-D74E-4C3F-9993-3836926AD336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F9D2EA-9C7D-4EFD-B1BD-49E93B52BFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
   <sheets>
     <sheet name="Model Iteration Log Filip" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="75">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -258,23 +258,35 @@
     <t>0.211</t>
   </si>
   <si>
-    <t>penalty='l2', loss='squared_hinge', C=2000.0, multi_class='ovr', fit_intercept=True, random_state=42, dual=True, max_iter=30000</t>
-  </si>
-  <si>
-    <t>0.262</t>
-  </si>
-  <si>
-    <t>0.206</t>
-  </si>
-  <si>
-    <t>0.214</t>
+    <t>SimpleRNN</t>
+  </si>
+  <si>
+    <t>keras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">features.py (baseline) + tf.keras.preprocessing.text.Tokenizer and tf.keras.preprocessing.sequence.pad_sequences </t>
+  </si>
+  <si>
+    <t>Sentence_Tok'</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>lr=1e-4, kernel_regularizer="l2" for the dense layers, batch_size=64</t>
+  </si>
+  <si>
+    <t>LSTM</t>
+  </si>
+  <si>
+    <t>lr=5e-3, kernel_regularizer="l2" for the dense layers, batch_size=64</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -343,6 +355,12 @@
       <name val="Aptos Display"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -506,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -583,6 +601,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -940,31 +961,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10A5CD43-FACF-4F92-BDE3-5E7B47D72998}">
   <dimension ref="B2:U51"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="6.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="6.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="36" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="32" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="33.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="31.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="20.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="33.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.33203125" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -986,31 +1007,31 @@
       <c r="T2" s="4"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="2:21" ht="24" x14ac:dyDescent="0.4">
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B3" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="28"/>
-      <c r="S3" s="28"/>
-      <c r="T3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="30"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -1031,18 +1052,18 @@
       <c r="S4" s="7"/>
       <c r="T4" s="8"/>
     </row>
-    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6"/>
       <c r="C5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -1054,18 +1075,18 @@
       <c r="S5" s="18"/>
       <c r="T5" s="19"/>
     </row>
-    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
       <c r="C6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
@@ -1077,7 +1098,7 @@
       <c r="S6" s="18"/>
       <c r="T6" s="19"/>
     </row>
-    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6"/>
       <c r="C7" s="18"/>
       <c r="D7" s="20"/>
@@ -1098,7 +1119,7 @@
       <c r="S7" s="18"/>
       <c r="T7" s="19"/>
     </row>
-    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6"/>
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
@@ -1119,34 +1140,34 @@
       <c r="S8" s="18"/>
       <c r="T8" s="19"/>
     </row>
-    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="16"/>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="31" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
       <c r="J9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="31" t="s">
+      <c r="K9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="31"/>
-      <c r="P9" s="30" t="s">
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="31"/>
       <c r="S9" s="22" t="s">
         <v>24</v>
       </c>
@@ -1154,7 +1175,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>7</v>
       </c>
@@ -1209,7 +1230,7 @@
       <c r="S10" s="25"/>
       <c r="T10" s="26"/>
     </row>
-    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="9">
         <v>1</v>
       </c>
@@ -1264,7 +1285,7 @@
       </c>
       <c r="T11" s="11"/>
     </row>
-    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>2</v>
       </c>
@@ -1315,7 +1336,7 @@
       </c>
       <c r="T12" s="11"/>
     </row>
-    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
         <v>3</v>
       </c>
@@ -1370,7 +1391,7 @@
       </c>
       <c r="T13" s="11"/>
     </row>
-    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="9">
         <v>4</v>
       </c>
@@ -1417,7 +1438,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="11"/>
     </row>
-    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="9">
         <v>5</v>
       </c>
@@ -1462,7 +1483,7 @@
       <c r="S15" s="10"/>
       <c r="T15" s="11"/>
     </row>
-    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="9">
         <v>6</v>
       </c>
@@ -1505,7 +1526,7 @@
       <c r="S16" s="10"/>
       <c r="T16" s="11"/>
     </row>
-    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="9">
         <v>7</v>
       </c>
@@ -1528,7 +1549,7 @@
       <c r="S17" s="10"/>
       <c r="T17" s="11"/>
     </row>
-    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9">
         <v>8</v>
       </c>
@@ -1551,7 +1572,7 @@
       <c r="S18" s="10"/>
       <c r="T18" s="11"/>
     </row>
-    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>9</v>
       </c>
@@ -1574,7 +1595,7 @@
       <c r="S19" s="10"/>
       <c r="T19" s="11"/>
     </row>
-    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="9">
         <v>10</v>
       </c>
@@ -1597,7 +1618,7 @@
       <c r="S20" s="10"/>
       <c r="T20" s="11"/>
     </row>
-    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9">
         <v>11</v>
       </c>
@@ -1620,7 +1641,7 @@
       <c r="S21" s="10"/>
       <c r="T21" s="11"/>
     </row>
-    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
         <v>12</v>
       </c>
@@ -1643,7 +1664,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="11"/>
     </row>
-    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
@@ -1666,7 +1687,7 @@
       <c r="S23" s="10"/>
       <c r="T23" s="11"/>
     </row>
-    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9">
         <v>14</v>
       </c>
@@ -1689,7 +1710,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="11"/>
     </row>
-    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9">
         <v>15</v>
       </c>
@@ -1712,7 +1733,7 @@
       <c r="S25" s="10"/>
       <c r="T25" s="11"/>
     </row>
-    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
         <v>16</v>
       </c>
@@ -1735,7 +1756,7 @@
       <c r="S26" s="10"/>
       <c r="T26" s="11"/>
     </row>
-    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="9">
         <v>17</v>
       </c>
@@ -1758,7 +1779,7 @@
       <c r="S27" s="10"/>
       <c r="T27" s="11"/>
     </row>
-    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="9">
         <v>18</v>
       </c>
@@ -1781,7 +1802,7 @@
       <c r="S28" s="10"/>
       <c r="T28" s="11"/>
     </row>
-    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="9">
         <v>19</v>
       </c>
@@ -1804,7 +1825,7 @@
       <c r="S29" s="10"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="9">
         <v>20</v>
       </c>
@@ -1827,7 +1848,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="11"/>
     </row>
-    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="9">
         <v>21</v>
       </c>
@@ -1850,7 +1871,7 @@
       <c r="S31" s="10"/>
       <c r="T31" s="11"/>
     </row>
-    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9">
         <v>22</v>
       </c>
@@ -1873,7 +1894,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="11"/>
     </row>
-    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="9">
         <v>23</v>
       </c>
@@ -1896,7 +1917,7 @@
       <c r="S33" s="10"/>
       <c r="T33" s="11"/>
     </row>
-    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="9">
         <v>24</v>
       </c>
@@ -1919,7 +1940,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="11"/>
     </row>
-    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="9">
         <v>25</v>
       </c>
@@ -1942,7 +1963,7 @@
       <c r="S35" s="10"/>
       <c r="T35" s="11"/>
     </row>
-    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9">
         <v>26</v>
       </c>
@@ -1965,7 +1986,7 @@
       <c r="S36" s="10"/>
       <c r="T36" s="11"/>
     </row>
-    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="9">
         <v>27</v>
       </c>
@@ -1988,7 +2009,7 @@
       <c r="S37" s="10"/>
       <c r="T37" s="11"/>
     </row>
-    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="9">
         <v>28</v>
       </c>
@@ -2011,7 +2032,7 @@
       <c r="S38" s="10"/>
       <c r="T38" s="11"/>
     </row>
-    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
         <v>29</v>
       </c>
@@ -2034,7 +2055,7 @@
       <c r="S39" s="10"/>
       <c r="T39" s="11"/>
     </row>
-    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9">
         <v>30</v>
       </c>
@@ -2057,7 +2078,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="11"/>
     </row>
-    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="9">
         <v>31</v>
       </c>
@@ -2080,7 +2101,7 @@
       <c r="S41" s="10"/>
       <c r="T41" s="11"/>
     </row>
-    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="9">
         <v>32</v>
       </c>
@@ -2103,7 +2124,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="11"/>
     </row>
-    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="9">
         <v>33</v>
       </c>
@@ -2126,7 +2147,7 @@
       <c r="S43" s="10"/>
       <c r="T43" s="11"/>
     </row>
-    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="9">
         <v>34</v>
       </c>
@@ -2149,7 +2170,7 @@
       <c r="S44" s="10"/>
       <c r="T44" s="11"/>
     </row>
-    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="9">
         <v>35</v>
       </c>
@@ -2172,7 +2193,7 @@
       <c r="S45" s="10"/>
       <c r="T45" s="11"/>
     </row>
-    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="9">
         <v>36</v>
       </c>
@@ -2195,7 +2216,7 @@
       <c r="S46" s="10"/>
       <c r="T46" s="11"/>
     </row>
-    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="9">
         <v>37</v>
       </c>
@@ -2218,7 +2239,7 @@
       <c r="S47" s="10"/>
       <c r="T47" s="11"/>
     </row>
-    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="9">
         <v>38</v>
       </c>
@@ -2241,7 +2262,7 @@
       <c r="S48" s="10"/>
       <c r="T48" s="11"/>
     </row>
-    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="9">
         <v>39</v>
       </c>
@@ -2264,7 +2285,7 @@
       <c r="S49" s="10"/>
       <c r="T49" s="11"/>
     </row>
-    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12">
         <v>40</v>
       </c>
@@ -2287,7 +2308,7 @@
       <c r="S50" s="13"/>
       <c r="T50" s="14"/>
     </row>
-    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C51" s="15" t="s">
         <v>8</v>
       </c>
@@ -2309,31 +2330,31 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F6E3FC4-92B9-4B14-9A38-1F80DD1D104A}">
   <dimension ref="B2:U51"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="6.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="6.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="36" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="32" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="33.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="31.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="20.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="33.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.33203125" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2355,31 +2376,31 @@
       <c r="T2" s="4"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="2:21" ht="24" x14ac:dyDescent="0.4">
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B3" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="28"/>
-      <c r="S3" s="28"/>
-      <c r="T3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="30"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -2400,18 +2421,18 @@
       <c r="S4" s="7"/>
       <c r="T4" s="8"/>
     </row>
-    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6"/>
       <c r="C5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -2423,18 +2444,18 @@
       <c r="S5" s="18"/>
       <c r="T5" s="19"/>
     </row>
-    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
       <c r="C6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
@@ -2446,7 +2467,7 @@
       <c r="S6" s="18"/>
       <c r="T6" s="19"/>
     </row>
-    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6"/>
       <c r="C7" s="18"/>
       <c r="D7" s="20"/>
@@ -2467,7 +2488,7 @@
       <c r="S7" s="18"/>
       <c r="T7" s="19"/>
     </row>
-    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6"/>
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
@@ -2488,34 +2509,34 @@
       <c r="S8" s="18"/>
       <c r="T8" s="19"/>
     </row>
-    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="16"/>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="31" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
       <c r="J9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="31" t="s">
+      <c r="K9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="31"/>
-      <c r="P9" s="30" t="s">
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="31"/>
       <c r="S9" s="22" t="s">
         <v>24</v>
       </c>
@@ -2523,7 +2544,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>7</v>
       </c>
@@ -2578,7 +2599,7 @@
       <c r="S10" s="25"/>
       <c r="T10" s="26"/>
     </row>
-    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="9">
         <v>1</v>
       </c>
@@ -2600,21 +2621,23 @@
       <c r="H11" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I11" s="10"/>
+      <c r="I11" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="J11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="K11" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="L11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="N11" s="10" t="s">
-        <v>50</v>
+      <c r="K11" s="10">
+        <v>0.24399999999999999</v>
+      </c>
+      <c r="L11" s="10">
+        <v>0.224</v>
+      </c>
+      <c r="M11" s="10">
+        <v>0.224</v>
+      </c>
+      <c r="N11" s="10">
+        <v>0.216</v>
       </c>
       <c r="O11" s="10"/>
       <c r="P11" s="10" t="s">
@@ -2631,7 +2654,7 @@
       </c>
       <c r="T11" s="11"/>
     </row>
-    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>2</v>
       </c>
@@ -2653,21 +2676,23 @@
       <c r="H12" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I12" s="10"/>
+      <c r="I12" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="J12" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="N12" s="10" t="s">
-        <v>53</v>
+      <c r="K12" s="10">
+        <v>0.29299999999999998</v>
+      </c>
+      <c r="L12" s="10">
+        <v>0.29099999999999998</v>
+      </c>
+      <c r="M12" s="10">
+        <v>0.29299999999999998</v>
+      </c>
+      <c r="N12" s="10">
+        <v>0.27400000000000002</v>
       </c>
       <c r="O12" s="10"/>
       <c r="P12" s="10" t="s">
@@ -2680,7 +2705,7 @@
       </c>
       <c r="T12" s="11"/>
     </row>
-    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
         <v>3</v>
       </c>
@@ -2702,21 +2727,23 @@
       <c r="H13" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I13" s="10"/>
+      <c r="I13" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="J13" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="K13" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="L13" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="N13" s="10" t="s">
-        <v>56</v>
+      <c r="K13" s="10">
+        <v>0.252</v>
+      </c>
+      <c r="L13" s="10">
+        <v>0.216</v>
+      </c>
+      <c r="M13" s="10">
+        <v>0.252</v>
+      </c>
+      <c r="N13" s="10">
+        <v>0.22</v>
       </c>
       <c r="O13" s="10"/>
       <c r="P13" s="10" t="s">
@@ -2733,7 +2760,7 @@
       </c>
       <c r="T13" s="11"/>
     </row>
-    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="9">
         <v>4</v>
       </c>
@@ -2755,21 +2782,23 @@
       <c r="H14" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="I14" s="10"/>
+      <c r="I14" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="J14" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="K14" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="M14" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="N14" s="10" t="s">
-        <v>57</v>
+      <c r="K14" s="10">
+        <v>0.248</v>
+      </c>
+      <c r="L14" s="10">
+        <v>0.22</v>
+      </c>
+      <c r="M14" s="10">
+        <v>0.248</v>
+      </c>
+      <c r="N14" s="10">
+        <v>0.219</v>
       </c>
       <c r="O14" s="10"/>
       <c r="P14" s="10"/>
@@ -2778,7 +2807,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="11"/>
     </row>
-    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="9">
         <v>5</v>
       </c>
@@ -2804,17 +2833,17 @@
       <c r="J15" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="K15" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="L15" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="N15" s="10" t="s">
-        <v>63</v>
+      <c r="K15" s="10">
+        <v>0.28699999999999998</v>
+      </c>
+      <c r="L15" s="10">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="M15" s="10">
+        <v>0.28699999999999998</v>
+      </c>
+      <c r="N15" s="10">
+        <v>0.23400000000000001</v>
       </c>
       <c r="O15" s="10"/>
       <c r="P15" s="10"/>
@@ -2823,7 +2852,7 @@
       <c r="S15" s="10"/>
       <c r="T15" s="11"/>
     </row>
-    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="9">
         <v>6</v>
       </c>
@@ -2842,24 +2871,22 @@
       <c r="G16" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="10" t="s">
-        <v>46</v>
-      </c>
+      <c r="H16" s="10"/>
       <c r="I16" s="10"/>
       <c r="J16" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="N16" s="10" t="s">
-        <v>70</v>
+        <v>42</v>
+      </c>
+      <c r="K16" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="L16" s="10">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="M16" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="N16" s="10">
+        <v>0.21099999999999999</v>
       </c>
       <c r="O16" s="10"/>
       <c r="P16" s="10"/>
@@ -2868,22 +2895,46 @@
       <c r="S16" s="10"/>
       <c r="T16" s="11"/>
     </row>
-    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="9">
         <v>7</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
+      <c r="C17" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="K17" s="10">
+        <v>0.56399999999999995</v>
+      </c>
+      <c r="L17" s="10">
+        <v>0.56499999999999995</v>
+      </c>
+      <c r="M17" s="10">
+        <v>0.56399999999999995</v>
+      </c>
+      <c r="N17" s="10">
+        <v>0.56299999999999994</v>
+      </c>
       <c r="O17" s="10"/>
       <c r="P17" s="10"/>
       <c r="Q17" s="10"/>
@@ -2891,22 +2942,46 @@
       <c r="S17" s="10"/>
       <c r="T17" s="11"/>
     </row>
-    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9">
         <v>8</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
+      <c r="C18" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H18" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="K18" s="10">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="L18" s="10">
+        <v>0.77800000000000002</v>
+      </c>
+      <c r="M18" s="10">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="N18" s="10">
+        <v>0.76700000000000002</v>
+      </c>
       <c r="O18" s="10"/>
       <c r="P18" s="10"/>
       <c r="Q18" s="10"/>
@@ -2914,7 +2989,7 @@
       <c r="S18" s="10"/>
       <c r="T18" s="11"/>
     </row>
-    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>9</v>
       </c>
@@ -2937,7 +3012,7 @@
       <c r="S19" s="10"/>
       <c r="T19" s="11"/>
     </row>
-    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="9">
         <v>10</v>
       </c>
@@ -2960,7 +3035,7 @@
       <c r="S20" s="10"/>
       <c r="T20" s="11"/>
     </row>
-    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9">
         <v>11</v>
       </c>
@@ -2983,7 +3058,7 @@
       <c r="S21" s="10"/>
       <c r="T21" s="11"/>
     </row>
-    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
         <v>12</v>
       </c>
@@ -3006,7 +3081,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="11"/>
     </row>
-    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
@@ -3029,7 +3104,7 @@
       <c r="S23" s="10"/>
       <c r="T23" s="11"/>
     </row>
-    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9">
         <v>14</v>
       </c>
@@ -3052,7 +3127,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="11"/>
     </row>
-    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9">
         <v>15</v>
       </c>
@@ -3075,7 +3150,7 @@
       <c r="S25" s="10"/>
       <c r="T25" s="11"/>
     </row>
-    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
         <v>16</v>
       </c>
@@ -3098,7 +3173,7 @@
       <c r="S26" s="10"/>
       <c r="T26" s="11"/>
     </row>
-    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="9">
         <v>17</v>
       </c>
@@ -3121,7 +3196,7 @@
       <c r="S27" s="10"/>
       <c r="T27" s="11"/>
     </row>
-    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="9">
         <v>18</v>
       </c>
@@ -3144,7 +3219,7 @@
       <c r="S28" s="10"/>
       <c r="T28" s="11"/>
     </row>
-    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="9">
         <v>19</v>
       </c>
@@ -3167,7 +3242,7 @@
       <c r="S29" s="10"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="9">
         <v>20</v>
       </c>
@@ -3190,7 +3265,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="11"/>
     </row>
-    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="9">
         <v>21</v>
       </c>
@@ -3213,7 +3288,7 @@
       <c r="S31" s="10"/>
       <c r="T31" s="11"/>
     </row>
-    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9">
         <v>22</v>
       </c>
@@ -3236,7 +3311,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="11"/>
     </row>
-    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="9">
         <v>23</v>
       </c>
@@ -3259,7 +3334,7 @@
       <c r="S33" s="10"/>
       <c r="T33" s="11"/>
     </row>
-    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="9">
         <v>24</v>
       </c>
@@ -3282,7 +3357,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="11"/>
     </row>
-    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="9">
         <v>25</v>
       </c>
@@ -3305,7 +3380,7 @@
       <c r="S35" s="10"/>
       <c r="T35" s="11"/>
     </row>
-    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9">
         <v>26</v>
       </c>
@@ -3328,7 +3403,7 @@
       <c r="S36" s="10"/>
       <c r="T36" s="11"/>
     </row>
-    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="9">
         <v>27</v>
       </c>
@@ -3351,7 +3426,7 @@
       <c r="S37" s="10"/>
       <c r="T37" s="11"/>
     </row>
-    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="9">
         <v>28</v>
       </c>
@@ -3374,7 +3449,7 @@
       <c r="S38" s="10"/>
       <c r="T38" s="11"/>
     </row>
-    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
         <v>29</v>
       </c>
@@ -3397,7 +3472,7 @@
       <c r="S39" s="10"/>
       <c r="T39" s="11"/>
     </row>
-    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9">
         <v>30</v>
       </c>
@@ -3420,7 +3495,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="11"/>
     </row>
-    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="9">
         <v>31</v>
       </c>
@@ -3443,7 +3518,7 @@
       <c r="S41" s="10"/>
       <c r="T41" s="11"/>
     </row>
-    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="9">
         <v>32</v>
       </c>
@@ -3466,7 +3541,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="11"/>
     </row>
-    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="9">
         <v>33</v>
       </c>
@@ -3489,7 +3564,7 @@
       <c r="S43" s="10"/>
       <c r="T43" s="11"/>
     </row>
-    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="9">
         <v>34</v>
       </c>
@@ -3512,7 +3587,7 @@
       <c r="S44" s="10"/>
       <c r="T44" s="11"/>
     </row>
-    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="9">
         <v>35</v>
       </c>
@@ -3535,7 +3610,7 @@
       <c r="S45" s="10"/>
       <c r="T45" s="11"/>
     </row>
-    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="9">
         <v>36</v>
       </c>
@@ -3558,7 +3633,7 @@
       <c r="S46" s="10"/>
       <c r="T46" s="11"/>
     </row>
-    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="9">
         <v>37</v>
       </c>
@@ -3581,7 +3656,7 @@
       <c r="S47" s="10"/>
       <c r="T47" s="11"/>
     </row>
-    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="9">
         <v>38</v>
       </c>
@@ -3604,7 +3679,7 @@
       <c r="S48" s="10"/>
       <c r="T48" s="11"/>
     </row>
-    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="9">
         <v>39</v>
       </c>
@@ -3627,7 +3702,7 @@
       <c r="S49" s="10"/>
       <c r="T49" s="11"/>
     </row>
-    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12">
         <v>40</v>
       </c>
@@ -3650,7 +3725,7 @@
       <c r="S50" s="13"/>
       <c r="T50" s="14"/>
     </row>
-    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C51" s="15" t="s">
         <v>8</v>
       </c>
@@ -3665,6 +3740,7 @@
     <mergeCell ref="K9:O9"/>
     <mergeCell ref="P9:R9"/>
   </mergeCells>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add saved models and update iteration log
This commit adds two saved keras models which are used in the Model
iterrations notebook to reproduce the performance described in the model
iteration file.
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\Documents\GitHub\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\git-school\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C7B153-6984-4FD3-9348-BC613535C898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05A80BF-B143-4C9E-B0E1-03860D18C7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
   <sheets>
     <sheet name="Model Iteration Log Filip" sheetId="1" r:id="rId1"/>
@@ -649,6 +649,81 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -658,92 +733,17 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1080,31 +1080,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10A5CD43-FACF-4F92-BDE3-5E7B47D72998}">
   <dimension ref="B2:U51"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="6.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="6.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="36" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="32" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="33.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="31.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="20.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="33.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.33203125" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -1126,31 +1126,31 @@
       <c r="T2" s="4"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="2:21" ht="24" x14ac:dyDescent="0.4">
-      <c r="B3" s="28" t="s">
+    <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B3" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="29"/>
-      <c r="R3" s="29"/>
-      <c r="S3" s="29"/>
-      <c r="T3" s="30"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="55"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -1171,18 +1171,18 @@
       <c r="S4" s="7"/>
       <c r="T4" s="8"/>
     </row>
-    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6"/>
       <c r="C5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -1194,18 +1194,18 @@
       <c r="S5" s="18"/>
       <c r="T5" s="19"/>
     </row>
-    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
       <c r="C6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="57"/>
+      <c r="J6" s="57"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
@@ -1217,7 +1217,7 @@
       <c r="S6" s="18"/>
       <c r="T6" s="19"/>
     </row>
-    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6"/>
       <c r="C7" s="18"/>
       <c r="D7" s="20"/>
@@ -1238,7 +1238,7 @@
       <c r="S7" s="18"/>
       <c r="T7" s="19"/>
     </row>
-    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6"/>
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
@@ -1259,50 +1259,50 @@
       <c r="S8" s="18"/>
       <c r="T8" s="19"/>
     </row>
-    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="35"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="35"/>
-      <c r="Q9" s="35"/>
-      <c r="R9" s="35"/>
-      <c r="S9" s="35"/>
-      <c r="T9" s="35"/>
-    </row>
-    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="35"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="37"/>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37"/>
-      <c r="K10" s="37"/>
-      <c r="L10" s="37"/>
-      <c r="M10" s="37"/>
-      <c r="N10" s="37"/>
-      <c r="O10" s="37"/>
-      <c r="P10" s="37"/>
-      <c r="Q10" s="37"/>
-      <c r="R10" s="37"/>
-      <c r="S10" s="37"/>
-      <c r="T10" s="37"/>
-    </row>
-    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="35"/>
+    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="28"/>
+      <c r="M9" s="28"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="28"/>
+      <c r="Q9" s="28"/>
+      <c r="R9" s="28"/>
+      <c r="S9" s="28"/>
+      <c r="T9" s="28"/>
+    </row>
+    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="28"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="30"/>
+      <c r="P10" s="30"/>
+      <c r="Q10" s="30"/>
+      <c r="R10" s="30"/>
+      <c r="S10" s="30"/>
+      <c r="T10" s="30"/>
+    </row>
+    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B11" s="28"/>
       <c r="C11" s="45" t="s">
         <v>0</v>
       </c>
@@ -1324,31 +1324,31 @@
       <c r="S11" s="46"/>
       <c r="T11" s="46"/>
     </row>
-    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="35"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="39"/>
-      <c r="L12" s="39"/>
-      <c r="M12" s="39"/>
-      <c r="N12" s="39"/>
-      <c r="O12" s="39"/>
-      <c r="P12" s="39"/>
-      <c r="Q12" s="39"/>
-      <c r="R12" s="39"/>
-      <c r="S12" s="39"/>
-      <c r="T12" s="39"/>
-    </row>
-    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="35"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="40" t="s">
+    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B12" s="28"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="32"/>
+      <c r="N12" s="32"/>
+      <c r="O12" s="32"/>
+      <c r="P12" s="32"/>
+      <c r="Q12" s="32"/>
+      <c r="R12" s="32"/>
+      <c r="S12" s="32"/>
+      <c r="T12" s="32"/>
+    </row>
+    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="28"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="33" t="s">
         <v>2</v>
       </c>
       <c r="E13" s="47"/>
@@ -1358,20 +1358,20 @@
       <c r="I13" s="47"/>
       <c r="J13" s="47"/>
       <c r="K13" s="47"/>
-      <c r="L13" s="40"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="40"/>
-      <c r="O13" s="40"/>
-      <c r="P13" s="40"/>
-      <c r="Q13" s="40"/>
-      <c r="R13" s="40"/>
-      <c r="S13" s="40"/>
-      <c r="T13" s="40"/>
-    </row>
-    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="35"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="40" t="s">
+      <c r="L13" s="33"/>
+      <c r="M13" s="33"/>
+      <c r="N13" s="33"/>
+      <c r="O13" s="33"/>
+      <c r="P13" s="33"/>
+      <c r="Q13" s="33"/>
+      <c r="R13" s="33"/>
+      <c r="S13" s="33"/>
+      <c r="T13" s="33"/>
+    </row>
+    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="28"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="33" t="s">
         <v>3</v>
       </c>
       <c r="E14" s="48"/>
@@ -1381,1079 +1381,1066 @@
       <c r="I14" s="48"/>
       <c r="J14" s="48"/>
       <c r="K14" s="48"/>
-      <c r="L14" s="40"/>
-      <c r="M14" s="40"/>
-      <c r="N14" s="40"/>
-      <c r="O14" s="40"/>
-      <c r="P14" s="40"/>
-      <c r="Q14" s="40"/>
-      <c r="R14" s="40"/>
-      <c r="S14" s="40"/>
-      <c r="T14" s="40"/>
-    </row>
-    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="35"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="40"/>
-      <c r="K15" s="40"/>
-      <c r="L15" s="40"/>
-      <c r="M15" s="40"/>
-      <c r="N15" s="40"/>
-      <c r="O15" s="40"/>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="40"/>
-      <c r="R15" s="40"/>
-      <c r="S15" s="40"/>
-      <c r="T15" s="40"/>
-    </row>
-    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="35"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="40"/>
-      <c r="K16" s="40"/>
-      <c r="L16" s="40"/>
-      <c r="M16" s="40"/>
-      <c r="N16" s="40"/>
-      <c r="O16" s="40"/>
-      <c r="P16" s="40"/>
-      <c r="Q16" s="40"/>
-      <c r="R16" s="40"/>
-      <c r="S16" s="40"/>
-      <c r="T16" s="40"/>
-    </row>
-    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="49"/>
-      <c r="C17" s="50"/>
-      <c r="D17" s="52" t="s">
+      <c r="L14" s="33"/>
+      <c r="M14" s="33"/>
+      <c r="N14" s="33"/>
+      <c r="O14" s="33"/>
+      <c r="P14" s="33"/>
+      <c r="Q14" s="33"/>
+      <c r="R14" s="33"/>
+      <c r="S14" s="33"/>
+      <c r="T14" s="33"/>
+    </row>
+    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="28"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+      <c r="J15" s="33"/>
+      <c r="K15" s="33"/>
+      <c r="L15" s="33"/>
+      <c r="M15" s="33"/>
+      <c r="N15" s="33"/>
+      <c r="O15" s="33"/>
+      <c r="P15" s="33"/>
+      <c r="Q15" s="33"/>
+      <c r="R15" s="33"/>
+      <c r="S15" s="33"/>
+      <c r="T15" s="33"/>
+    </row>
+    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="28"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+      <c r="P16" s="33"/>
+      <c r="Q16" s="33"/>
+      <c r="R16" s="33"/>
+      <c r="S16" s="33"/>
+      <c r="T16" s="33"/>
+    </row>
+    <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="42"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="52"/>
-      <c r="F17" s="54" t="s">
+      <c r="E17" s="50"/>
+      <c r="F17" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="G17" s="54"/>
-      <c r="H17" s="54"/>
-      <c r="I17" s="54"/>
-      <c r="J17" s="54"/>
-      <c r="K17" s="52" t="s">
+      <c r="G17" s="51"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="L17" s="54" t="s">
+      <c r="L17" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="M17" s="54"/>
-      <c r="N17" s="54"/>
-      <c r="O17" s="54"/>
-      <c r="P17" s="54"/>
-      <c r="Q17" s="52" t="s">
+      <c r="M17" s="51"/>
+      <c r="N17" s="51"/>
+      <c r="O17" s="51"/>
+      <c r="P17" s="51"/>
+      <c r="Q17" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="R17" s="52"/>
-      <c r="S17" s="52"/>
-      <c r="T17" s="54" t="s">
+      <c r="R17" s="50"/>
+      <c r="S17" s="50"/>
+      <c r="T17" s="51" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="49"/>
-      <c r="C18" s="51"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="53"/>
-      <c r="L18" s="56" t="s">
+    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="42"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="41"/>
+      <c r="L18" s="52" t="s">
         <v>60</v>
       </c>
-      <c r="M18" s="56"/>
-      <c r="N18" s="56"/>
-      <c r="O18" s="56"/>
-      <c r="P18" s="56"/>
-      <c r="Q18" s="53"/>
-      <c r="R18" s="53"/>
-      <c r="S18" s="53"/>
-      <c r="T18" s="55"/>
-    </row>
-    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="49"/>
-      <c r="C19" s="57" t="s">
+      <c r="M18" s="52"/>
+      <c r="N18" s="52"/>
+      <c r="O18" s="52"/>
+      <c r="P18" s="52"/>
+      <c r="Q18" s="41"/>
+      <c r="R18" s="41"/>
+      <c r="S18" s="41"/>
+      <c r="T18" s="39"/>
+    </row>
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="42"/>
+      <c r="C19" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="58" t="s">
+      <c r="D19" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="58" t="s">
+      <c r="E19" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="F19" s="59" t="s">
+      <c r="F19" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="G19" s="59" t="s">
+      <c r="G19" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="59" t="s">
+      <c r="H19" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="I19" s="41" t="s">
+      <c r="I19" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="J19" s="41" t="s">
+      <c r="J19" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="K19" s="58" t="s">
+      <c r="K19" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="L19" s="59" t="s">
+      <c r="L19" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="M19" s="59" t="s">
+      <c r="M19" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="N19" s="59" t="s">
+      <c r="N19" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="O19" s="59" t="s">
+      <c r="O19" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="P19" s="41" t="s">
+      <c r="P19" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="Q19" s="58" t="s">
+      <c r="Q19" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="R19" s="58" t="s">
+      <c r="R19" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="S19" s="58" t="s">
+      <c r="S19" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="T19" s="59"/>
-    </row>
-    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="49"/>
-      <c r="C20" s="51"/>
-      <c r="D20" s="53"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="42" t="s">
+      <c r="T19" s="38"/>
+    </row>
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="42"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="J20" s="42" t="s">
+      <c r="J20" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="K20" s="53"/>
-      <c r="L20" s="55"/>
-      <c r="M20" s="55"/>
-      <c r="N20" s="55"/>
-      <c r="O20" s="55"/>
-      <c r="P20" s="42" t="s">
+      <c r="K20" s="41"/>
+      <c r="L20" s="39"/>
+      <c r="M20" s="39"/>
+      <c r="N20" s="39"/>
+      <c r="O20" s="39"/>
+      <c r="P20" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="Q20" s="53"/>
-      <c r="R20" s="53"/>
-      <c r="S20" s="53"/>
-      <c r="T20" s="55"/>
-    </row>
-    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="35"/>
-      <c r="C21" s="43">
+      <c r="Q20" s="41"/>
+      <c r="R20" s="41"/>
+      <c r="S20" s="41"/>
+      <c r="T20" s="39"/>
+    </row>
+    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="28"/>
+      <c r="C21" s="36">
         <v>1</v>
       </c>
-      <c r="D21" s="44" t="s">
+      <c r="D21" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="44" t="s">
+      <c r="E21" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="44" t="s">
+      <c r="F21" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G21" s="44" t="s">
+      <c r="G21" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H21" s="44" t="s">
+      <c r="H21" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="I21" s="44" t="s">
+      <c r="I21" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="44"/>
-      <c r="K21" s="44" t="s">
+      <c r="J21" s="37"/>
+      <c r="K21" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="L21" s="44">
+      <c r="L21" s="37">
         <v>0.24399999999999999</v>
       </c>
-      <c r="M21" s="44">
+      <c r="M21" s="37">
         <v>0.224</v>
       </c>
-      <c r="N21" s="44">
+      <c r="N21" s="37">
         <v>0.224</v>
       </c>
-      <c r="O21" s="44">
+      <c r="O21" s="37">
         <v>0.216</v>
       </c>
-      <c r="P21" s="44"/>
-      <c r="Q21" s="44" t="s">
+      <c r="P21" s="37"/>
+      <c r="Q21" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="R21" s="44" t="s">
+      <c r="R21" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="S21" s="44" t="s">
+      <c r="S21" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="T21" s="44" t="s">
+      <c r="T21" s="37" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="35"/>
-      <c r="C22" s="43">
+    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="28"/>
+      <c r="C22" s="36">
         <v>2</v>
       </c>
-      <c r="D22" s="44" t="s">
+      <c r="D22" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="44" t="s">
+      <c r="E22" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F22" s="44" t="s">
+      <c r="F22" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G22" s="44" t="s">
+      <c r="G22" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="44" t="s">
+      <c r="H22" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="I22" s="44" t="s">
+      <c r="I22" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="J22" s="44"/>
-      <c r="K22" s="44" t="s">
+      <c r="J22" s="37"/>
+      <c r="K22" s="37" t="s">
         <v>40</v>
       </c>
-      <c r="L22" s="44">
+      <c r="L22" s="37">
         <v>0.29299999999999998</v>
       </c>
-      <c r="M22" s="44">
+      <c r="M22" s="37">
         <v>0.29099999999999998</v>
       </c>
-      <c r="N22" s="44">
+      <c r="N22" s="37">
         <v>0.29299999999999998</v>
       </c>
-      <c r="O22" s="44">
+      <c r="O22" s="37">
         <v>0.27400000000000002</v>
       </c>
-      <c r="P22" s="44"/>
-      <c r="Q22" s="44" t="s">
+      <c r="P22" s="37"/>
+      <c r="Q22" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="R22" s="44"/>
-      <c r="S22" s="44"/>
-      <c r="T22" s="44" t="s">
+      <c r="R22" s="37"/>
+      <c r="S22" s="37"/>
+      <c r="T22" s="37" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="35"/>
-      <c r="C23" s="43">
+    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="28"/>
+      <c r="C23" s="36">
         <v>3</v>
       </c>
-      <c r="D23" s="44" t="s">
+      <c r="D23" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E23" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="44" t="s">
+      <c r="F23" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G23" s="44" t="s">
+      <c r="G23" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H23" s="44" t="s">
+      <c r="H23" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="I23" s="44" t="s">
+      <c r="I23" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="J23" s="44"/>
-      <c r="K23" s="44" t="s">
+      <c r="J23" s="37"/>
+      <c r="K23" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="L23" s="44">
+      <c r="L23" s="37">
         <v>0.252</v>
       </c>
-      <c r="M23" s="44">
+      <c r="M23" s="37">
         <v>0.216</v>
       </c>
-      <c r="N23" s="44">
+      <c r="N23" s="37">
         <v>0.252</v>
       </c>
-      <c r="O23" s="44">
+      <c r="O23" s="37">
         <v>0.22</v>
       </c>
-      <c r="P23" s="44"/>
-      <c r="Q23" s="44" t="s">
+      <c r="P23" s="37"/>
+      <c r="Q23" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="R23" s="44" t="s">
+      <c r="R23" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="S23" s="44" t="s">
+      <c r="S23" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="T23" s="44" t="s">
+      <c r="T23" s="37" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="35"/>
-      <c r="C24" s="43">
+    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="28"/>
+      <c r="C24" s="36">
         <v>4</v>
       </c>
-      <c r="D24" s="44" t="s">
+      <c r="D24" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="44" t="s">
+      <c r="E24" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F24" s="44" t="s">
+      <c r="F24" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G24" s="44" t="s">
+      <c r="G24" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H24" s="44" t="s">
+      <c r="H24" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="I24" s="44" t="s">
+      <c r="I24" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="J24" s="44"/>
-      <c r="K24" s="44" t="s">
+      <c r="J24" s="37"/>
+      <c r="K24" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="L24" s="44">
+      <c r="L24" s="37">
         <v>0.248</v>
       </c>
-      <c r="M24" s="44">
+      <c r="M24" s="37">
         <v>0.22</v>
       </c>
-      <c r="N24" s="44">
+      <c r="N24" s="37">
         <v>0.248</v>
       </c>
-      <c r="O24" s="44">
+      <c r="O24" s="37">
         <v>0.219</v>
       </c>
-      <c r="P24" s="44"/>
-      <c r="Q24" s="44"/>
-      <c r="R24" s="44"/>
-      <c r="S24" s="44"/>
-      <c r="T24" s="44"/>
-    </row>
-    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="35"/>
-      <c r="C25" s="43">
+      <c r="P24" s="37"/>
+      <c r="Q24" s="37"/>
+      <c r="R24" s="37"/>
+      <c r="S24" s="37"/>
+      <c r="T24" s="37"/>
+    </row>
+    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="28"/>
+      <c r="C25" s="36">
         <v>5</v>
       </c>
-      <c r="D25" s="44" t="s">
+      <c r="D25" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E25" s="44" t="s">
+      <c r="E25" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F25" s="44" t="s">
+      <c r="F25" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G25" s="44" t="s">
+      <c r="G25" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H25" s="44" t="s">
+      <c r="H25" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="I25" s="44" t="s">
+      <c r="I25" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="J25" s="44"/>
-      <c r="K25" s="44" t="s">
+      <c r="J25" s="37"/>
+      <c r="K25" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="L25" s="44">
+      <c r="L25" s="37">
         <v>0.28699999999999998</v>
       </c>
-      <c r="M25" s="44">
+      <c r="M25" s="37">
         <v>0.23300000000000001</v>
       </c>
-      <c r="N25" s="44">
+      <c r="N25" s="37">
         <v>0.28699999999999998</v>
       </c>
-      <c r="O25" s="44">
+      <c r="O25" s="37">
         <v>0.23400000000000001</v>
       </c>
-      <c r="P25" s="44"/>
-      <c r="Q25" s="44"/>
-      <c r="R25" s="44"/>
-      <c r="S25" s="44"/>
-      <c r="T25" s="44"/>
-    </row>
-    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="35"/>
-      <c r="C26" s="43">
+      <c r="P25" s="37"/>
+      <c r="Q25" s="37"/>
+      <c r="R25" s="37"/>
+      <c r="S25" s="37"/>
+      <c r="T25" s="37"/>
+    </row>
+    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="28"/>
+      <c r="C26" s="36">
         <v>6</v>
       </c>
-      <c r="D26" s="44" t="s">
+      <c r="D26" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E26" s="44" t="s">
+      <c r="E26" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F26" s="44" t="s">
+      <c r="F26" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G26" s="44" t="s">
+      <c r="G26" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H26" s="44" t="s">
+      <c r="H26" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="I26" s="44" t="s">
+      <c r="I26" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="J26" s="44"/>
-      <c r="K26" s="44" t="s">
+      <c r="J26" s="37"/>
+      <c r="K26" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="L26" s="44">
+      <c r="L26" s="37">
         <v>0.26200000000000001</v>
       </c>
-      <c r="M26" s="44">
+      <c r="M26" s="37">
         <v>0.20599999999999999</v>
       </c>
-      <c r="N26" s="44">
+      <c r="N26" s="37">
         <v>0.26200000000000001</v>
       </c>
-      <c r="O26" s="44">
+      <c r="O26" s="37">
         <v>0.214</v>
       </c>
-      <c r="P26" s="44"/>
-      <c r="Q26" s="44"/>
-      <c r="R26" s="44"/>
-      <c r="S26" s="44"/>
-      <c r="T26" s="44"/>
-    </row>
-    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="35"/>
-      <c r="C27" s="43">
+      <c r="P26" s="37"/>
+      <c r="Q26" s="37"/>
+      <c r="R26" s="37"/>
+      <c r="S26" s="37"/>
+      <c r="T26" s="37"/>
+    </row>
+    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="28"/>
+      <c r="C27" s="36">
         <v>7</v>
       </c>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="44"/>
-      <c r="I27" s="44"/>
-      <c r="J27" s="44"/>
-      <c r="K27" s="44"/>
-      <c r="L27" s="44"/>
-      <c r="M27" s="44"/>
-      <c r="N27" s="44"/>
-      <c r="O27" s="44"/>
-      <c r="P27" s="44"/>
-      <c r="Q27" s="44"/>
-      <c r="R27" s="44"/>
-      <c r="S27" s="44"/>
-      <c r="T27" s="44"/>
-    </row>
-    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="35"/>
-      <c r="C28" s="43">
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="37"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="37"/>
+      <c r="M27" s="37"/>
+      <c r="N27" s="37"/>
+      <c r="O27" s="37"/>
+      <c r="P27" s="37"/>
+      <c r="Q27" s="37"/>
+      <c r="R27" s="37"/>
+      <c r="S27" s="37"/>
+      <c r="T27" s="37"/>
+    </row>
+    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="28"/>
+      <c r="C28" s="36">
         <v>8</v>
       </c>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44"/>
-      <c r="F28" s="44"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="44"/>
-      <c r="I28" s="44"/>
-      <c r="J28" s="44"/>
-      <c r="K28" s="44"/>
-      <c r="L28" s="44"/>
-      <c r="M28" s="44"/>
-      <c r="N28" s="44"/>
-      <c r="O28" s="44"/>
-      <c r="P28" s="44"/>
-      <c r="Q28" s="44"/>
-      <c r="R28" s="44"/>
-      <c r="S28" s="44"/>
-      <c r="T28" s="44"/>
-    </row>
-    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="35"/>
-      <c r="C29" s="43">
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="37"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="37"/>
+      <c r="M28" s="37"/>
+      <c r="N28" s="37"/>
+      <c r="O28" s="37"/>
+      <c r="P28" s="37"/>
+      <c r="Q28" s="37"/>
+      <c r="R28" s="37"/>
+      <c r="S28" s="37"/>
+      <c r="T28" s="37"/>
+    </row>
+    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="28"/>
+      <c r="C29" s="36">
         <v>9</v>
       </c>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="44"/>
-      <c r="J29" s="44"/>
-      <c r="K29" s="44"/>
-      <c r="L29" s="44"/>
-      <c r="M29" s="44"/>
-      <c r="N29" s="44"/>
-      <c r="O29" s="44"/>
-      <c r="P29" s="44"/>
-      <c r="Q29" s="44"/>
-      <c r="R29" s="44"/>
-      <c r="S29" s="44"/>
-      <c r="T29" s="44"/>
-    </row>
-    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="35"/>
-      <c r="C30" s="43">
+      <c r="D29" s="37"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="37"/>
+      <c r="I29" s="37"/>
+      <c r="J29" s="37"/>
+      <c r="K29" s="37"/>
+      <c r="L29" s="37"/>
+      <c r="M29" s="37"/>
+      <c r="N29" s="37"/>
+      <c r="O29" s="37"/>
+      <c r="P29" s="37"/>
+      <c r="Q29" s="37"/>
+      <c r="R29" s="37"/>
+      <c r="S29" s="37"/>
+      <c r="T29" s="37"/>
+    </row>
+    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="28"/>
+      <c r="C30" s="36">
         <v>10</v>
       </c>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44"/>
-      <c r="K30" s="44"/>
-      <c r="L30" s="44"/>
-      <c r="M30" s="44"/>
-      <c r="N30" s="44"/>
-      <c r="O30" s="44"/>
-      <c r="P30" s="44"/>
-      <c r="Q30" s="44"/>
-      <c r="R30" s="44"/>
-      <c r="S30" s="44"/>
-      <c r="T30" s="44"/>
-    </row>
-    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="35"/>
-      <c r="C31" s="43">
+      <c r="D30" s="37"/>
+      <c r="E30" s="37"/>
+      <c r="F30" s="37"/>
+      <c r="G30" s="37"/>
+      <c r="H30" s="37"/>
+      <c r="I30" s="37"/>
+      <c r="J30" s="37"/>
+      <c r="K30" s="37"/>
+      <c r="L30" s="37"/>
+      <c r="M30" s="37"/>
+      <c r="N30" s="37"/>
+      <c r="O30" s="37"/>
+      <c r="P30" s="37"/>
+      <c r="Q30" s="37"/>
+      <c r="R30" s="37"/>
+      <c r="S30" s="37"/>
+      <c r="T30" s="37"/>
+    </row>
+    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="28"/>
+      <c r="C31" s="36">
         <v>11</v>
       </c>
-      <c r="D31" s="44"/>
-      <c r="E31" s="44"/>
-      <c r="F31" s="44"/>
-      <c r="G31" s="44"/>
-      <c r="H31" s="44"/>
-      <c r="I31" s="44"/>
-      <c r="J31" s="44"/>
-      <c r="K31" s="44"/>
-      <c r="L31" s="44"/>
-      <c r="M31" s="44"/>
-      <c r="N31" s="44"/>
-      <c r="O31" s="44"/>
-      <c r="P31" s="44"/>
-      <c r="Q31" s="44"/>
-      <c r="R31" s="44"/>
-      <c r="S31" s="44"/>
-      <c r="T31" s="44"/>
-    </row>
-    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="35"/>
-      <c r="C32" s="43">
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="37"/>
+      <c r="K31" s="37"/>
+      <c r="L31" s="37"/>
+      <c r="M31" s="37"/>
+      <c r="N31" s="37"/>
+      <c r="O31" s="37"/>
+      <c r="P31" s="37"/>
+      <c r="Q31" s="37"/>
+      <c r="R31" s="37"/>
+      <c r="S31" s="37"/>
+      <c r="T31" s="37"/>
+    </row>
+    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="28"/>
+      <c r="C32" s="36">
         <v>12</v>
       </c>
-      <c r="D32" s="44"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44"/>
-      <c r="J32" s="44"/>
-      <c r="K32" s="44"/>
-      <c r="L32" s="44"/>
-      <c r="M32" s="44"/>
-      <c r="N32" s="44"/>
-      <c r="O32" s="44"/>
-      <c r="P32" s="44"/>
-      <c r="Q32" s="44"/>
-      <c r="R32" s="44"/>
-      <c r="S32" s="44"/>
-      <c r="T32" s="44"/>
-    </row>
-    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="35"/>
-      <c r="C33" s="43">
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="37"/>
+      <c r="K32" s="37"/>
+      <c r="L32" s="37"/>
+      <c r="M32" s="37"/>
+      <c r="N32" s="37"/>
+      <c r="O32" s="37"/>
+      <c r="P32" s="37"/>
+      <c r="Q32" s="37"/>
+      <c r="R32" s="37"/>
+      <c r="S32" s="37"/>
+      <c r="T32" s="37"/>
+    </row>
+    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="28"/>
+      <c r="C33" s="36">
         <v>13</v>
       </c>
-      <c r="D33" s="44"/>
-      <c r="E33" s="44"/>
-      <c r="F33" s="44"/>
-      <c r="G33" s="44"/>
-      <c r="H33" s="44"/>
-      <c r="I33" s="44"/>
-      <c r="J33" s="44"/>
-      <c r="K33" s="44"/>
-      <c r="L33" s="44"/>
-      <c r="M33" s="44"/>
-      <c r="N33" s="44"/>
-      <c r="O33" s="44"/>
-      <c r="P33" s="44"/>
-      <c r="Q33" s="44"/>
-      <c r="R33" s="44"/>
-      <c r="S33" s="44"/>
-      <c r="T33" s="44"/>
-    </row>
-    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="35"/>
-      <c r="C34" s="43">
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="37"/>
+      <c r="K33" s="37"/>
+      <c r="L33" s="37"/>
+      <c r="M33" s="37"/>
+      <c r="N33" s="37"/>
+      <c r="O33" s="37"/>
+      <c r="P33" s="37"/>
+      <c r="Q33" s="37"/>
+      <c r="R33" s="37"/>
+      <c r="S33" s="37"/>
+      <c r="T33" s="37"/>
+    </row>
+    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="28"/>
+      <c r="C34" s="36">
         <v>14</v>
       </c>
-      <c r="D34" s="44"/>
-      <c r="E34" s="44"/>
-      <c r="F34" s="44"/>
-      <c r="G34" s="44"/>
-      <c r="H34" s="44"/>
-      <c r="I34" s="44"/>
-      <c r="J34" s="44"/>
-      <c r="K34" s="44"/>
-      <c r="L34" s="44"/>
-      <c r="M34" s="44"/>
-      <c r="N34" s="44"/>
-      <c r="O34" s="44"/>
-      <c r="P34" s="44"/>
-      <c r="Q34" s="44"/>
-      <c r="R34" s="44"/>
-      <c r="S34" s="44"/>
-      <c r="T34" s="44"/>
-    </row>
-    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="35"/>
-      <c r="C35" s="43">
+      <c r="D34" s="37"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="37"/>
+      <c r="K34" s="37"/>
+      <c r="L34" s="37"/>
+      <c r="M34" s="37"/>
+      <c r="N34" s="37"/>
+      <c r="O34" s="37"/>
+      <c r="P34" s="37"/>
+      <c r="Q34" s="37"/>
+      <c r="R34" s="37"/>
+      <c r="S34" s="37"/>
+      <c r="T34" s="37"/>
+    </row>
+    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="28"/>
+      <c r="C35" s="36">
         <v>15</v>
       </c>
-      <c r="D35" s="44"/>
-      <c r="E35" s="44"/>
-      <c r="F35" s="44"/>
-      <c r="G35" s="44"/>
-      <c r="H35" s="44"/>
-      <c r="I35" s="44"/>
-      <c r="J35" s="44"/>
-      <c r="K35" s="44"/>
-      <c r="L35" s="44"/>
-      <c r="M35" s="44"/>
-      <c r="N35" s="44"/>
-      <c r="O35" s="44"/>
-      <c r="P35" s="44"/>
-      <c r="Q35" s="44"/>
-      <c r="R35" s="44"/>
-      <c r="S35" s="44"/>
-      <c r="T35" s="44"/>
-    </row>
-    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="35"/>
-      <c r="C36" s="43">
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="37"/>
+      <c r="K35" s="37"/>
+      <c r="L35" s="37"/>
+      <c r="M35" s="37"/>
+      <c r="N35" s="37"/>
+      <c r="O35" s="37"/>
+      <c r="P35" s="37"/>
+      <c r="Q35" s="37"/>
+      <c r="R35" s="37"/>
+      <c r="S35" s="37"/>
+      <c r="T35" s="37"/>
+    </row>
+    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="28"/>
+      <c r="C36" s="36">
         <v>16</v>
       </c>
-      <c r="D36" s="44"/>
-      <c r="E36" s="44"/>
-      <c r="F36" s="44"/>
-      <c r="G36" s="44"/>
-      <c r="H36" s="44"/>
-      <c r="I36" s="44"/>
-      <c r="J36" s="44"/>
-      <c r="K36" s="44"/>
-      <c r="L36" s="44"/>
-      <c r="M36" s="44"/>
-      <c r="N36" s="44"/>
-      <c r="O36" s="44"/>
-      <c r="P36" s="44"/>
-      <c r="Q36" s="44"/>
-      <c r="R36" s="44"/>
-      <c r="S36" s="44"/>
-      <c r="T36" s="44"/>
-    </row>
-    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="35"/>
-      <c r="C37" s="43">
+      <c r="D36" s="37"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="37"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="37"/>
+      <c r="I36" s="37"/>
+      <c r="J36" s="37"/>
+      <c r="K36" s="37"/>
+      <c r="L36" s="37"/>
+      <c r="M36" s="37"/>
+      <c r="N36" s="37"/>
+      <c r="O36" s="37"/>
+      <c r="P36" s="37"/>
+      <c r="Q36" s="37"/>
+      <c r="R36" s="37"/>
+      <c r="S36" s="37"/>
+      <c r="T36" s="37"/>
+    </row>
+    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="28"/>
+      <c r="C37" s="36">
         <v>17</v>
       </c>
-      <c r="D37" s="44"/>
-      <c r="E37" s="44"/>
-      <c r="F37" s="44"/>
-      <c r="G37" s="44"/>
-      <c r="H37" s="44"/>
-      <c r="I37" s="44"/>
-      <c r="J37" s="44"/>
-      <c r="K37" s="44"/>
-      <c r="L37" s="44"/>
-      <c r="M37" s="44"/>
-      <c r="N37" s="44"/>
-      <c r="O37" s="44"/>
-      <c r="P37" s="44"/>
-      <c r="Q37" s="44"/>
-      <c r="R37" s="44"/>
-      <c r="S37" s="44"/>
-      <c r="T37" s="44"/>
-    </row>
-    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="35"/>
-      <c r="C38" s="43">
+      <c r="D37" s="37"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="37"/>
+      <c r="I37" s="37"/>
+      <c r="J37" s="37"/>
+      <c r="K37" s="37"/>
+      <c r="L37" s="37"/>
+      <c r="M37" s="37"/>
+      <c r="N37" s="37"/>
+      <c r="O37" s="37"/>
+      <c r="P37" s="37"/>
+      <c r="Q37" s="37"/>
+      <c r="R37" s="37"/>
+      <c r="S37" s="37"/>
+      <c r="T37" s="37"/>
+    </row>
+    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="28"/>
+      <c r="C38" s="36">
         <v>18</v>
       </c>
-      <c r="D38" s="44"/>
-      <c r="E38" s="44"/>
-      <c r="F38" s="44"/>
-      <c r="G38" s="44"/>
-      <c r="H38" s="44"/>
-      <c r="I38" s="44"/>
-      <c r="J38" s="44"/>
-      <c r="K38" s="44"/>
-      <c r="L38" s="44"/>
-      <c r="M38" s="44"/>
-      <c r="N38" s="44"/>
-      <c r="O38" s="44"/>
-      <c r="P38" s="44"/>
-      <c r="Q38" s="44"/>
-      <c r="R38" s="44"/>
-      <c r="S38" s="44"/>
-      <c r="T38" s="44"/>
-    </row>
-    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="35"/>
-      <c r="C39" s="43">
+      <c r="D38" s="37"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="37"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="37"/>
+      <c r="I38" s="37"/>
+      <c r="J38" s="37"/>
+      <c r="K38" s="37"/>
+      <c r="L38" s="37"/>
+      <c r="M38" s="37"/>
+      <c r="N38" s="37"/>
+      <c r="O38" s="37"/>
+      <c r="P38" s="37"/>
+      <c r="Q38" s="37"/>
+      <c r="R38" s="37"/>
+      <c r="S38" s="37"/>
+      <c r="T38" s="37"/>
+    </row>
+    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="28"/>
+      <c r="C39" s="36">
         <v>19</v>
       </c>
-      <c r="D39" s="44"/>
-      <c r="E39" s="44"/>
-      <c r="F39" s="44"/>
-      <c r="G39" s="44"/>
-      <c r="H39" s="44"/>
-      <c r="I39" s="44"/>
-      <c r="J39" s="44"/>
-      <c r="K39" s="44"/>
-      <c r="L39" s="44"/>
-      <c r="M39" s="44"/>
-      <c r="N39" s="44"/>
-      <c r="O39" s="44"/>
-      <c r="P39" s="44"/>
-      <c r="Q39" s="44"/>
-      <c r="R39" s="44"/>
-      <c r="S39" s="44"/>
-      <c r="T39" s="44"/>
-    </row>
-    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="35"/>
-      <c r="C40" s="43">
+      <c r="D39" s="37"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="37"/>
+      <c r="I39" s="37"/>
+      <c r="J39" s="37"/>
+      <c r="K39" s="37"/>
+      <c r="L39" s="37"/>
+      <c r="M39" s="37"/>
+      <c r="N39" s="37"/>
+      <c r="O39" s="37"/>
+      <c r="P39" s="37"/>
+      <c r="Q39" s="37"/>
+      <c r="R39" s="37"/>
+      <c r="S39" s="37"/>
+      <c r="T39" s="37"/>
+    </row>
+    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="28"/>
+      <c r="C40" s="36">
         <v>20</v>
       </c>
-      <c r="D40" s="44"/>
-      <c r="E40" s="44"/>
-      <c r="F40" s="44"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="44"/>
-      <c r="I40" s="44"/>
-      <c r="J40" s="44"/>
-      <c r="K40" s="44"/>
-      <c r="L40" s="44"/>
-      <c r="M40" s="44"/>
-      <c r="N40" s="44"/>
-      <c r="O40" s="44"/>
-      <c r="P40" s="44"/>
-      <c r="Q40" s="44"/>
-      <c r="R40" s="44"/>
-      <c r="S40" s="44"/>
-      <c r="T40" s="44"/>
-    </row>
-    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="35"/>
-      <c r="C41" s="43">
+      <c r="D40" s="37"/>
+      <c r="E40" s="37"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="37"/>
+      <c r="I40" s="37"/>
+      <c r="J40" s="37"/>
+      <c r="K40" s="37"/>
+      <c r="L40" s="37"/>
+      <c r="M40" s="37"/>
+      <c r="N40" s="37"/>
+      <c r="O40" s="37"/>
+      <c r="P40" s="37"/>
+      <c r="Q40" s="37"/>
+      <c r="R40" s="37"/>
+      <c r="S40" s="37"/>
+      <c r="T40" s="37"/>
+    </row>
+    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="28"/>
+      <c r="C41" s="36">
         <v>21</v>
       </c>
-      <c r="D41" s="44"/>
-      <c r="E41" s="44"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="44"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="44"/>
-      <c r="J41" s="44"/>
-      <c r="K41" s="44"/>
-      <c r="L41" s="44"/>
-      <c r="M41" s="44"/>
-      <c r="N41" s="44"/>
-      <c r="O41" s="44"/>
-      <c r="P41" s="44"/>
-      <c r="Q41" s="44"/>
-      <c r="R41" s="44"/>
-      <c r="S41" s="44"/>
-      <c r="T41" s="44"/>
-    </row>
-    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="35"/>
-      <c r="C42" s="43">
+      <c r="D41" s="37"/>
+      <c r="E41" s="37"/>
+      <c r="F41" s="37"/>
+      <c r="G41" s="37"/>
+      <c r="H41" s="37"/>
+      <c r="I41" s="37"/>
+      <c r="J41" s="37"/>
+      <c r="K41" s="37"/>
+      <c r="L41" s="37"/>
+      <c r="M41" s="37"/>
+      <c r="N41" s="37"/>
+      <c r="O41" s="37"/>
+      <c r="P41" s="37"/>
+      <c r="Q41" s="37"/>
+      <c r="R41" s="37"/>
+      <c r="S41" s="37"/>
+      <c r="T41" s="37"/>
+    </row>
+    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="28"/>
+      <c r="C42" s="36">
         <v>22</v>
       </c>
-      <c r="D42" s="44"/>
-      <c r="E42" s="44"/>
-      <c r="F42" s="44"/>
-      <c r="G42" s="44"/>
-      <c r="H42" s="44"/>
-      <c r="I42" s="44"/>
-      <c r="J42" s="44"/>
-      <c r="K42" s="44"/>
-      <c r="L42" s="44"/>
-      <c r="M42" s="44"/>
-      <c r="N42" s="44"/>
-      <c r="O42" s="44"/>
-      <c r="P42" s="44"/>
-      <c r="Q42" s="44"/>
-      <c r="R42" s="44"/>
-      <c r="S42" s="44"/>
-      <c r="T42" s="44"/>
-    </row>
-    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="35"/>
-      <c r="C43" s="43">
+      <c r="D42" s="37"/>
+      <c r="E42" s="37"/>
+      <c r="F42" s="37"/>
+      <c r="G42" s="37"/>
+      <c r="H42" s="37"/>
+      <c r="I42" s="37"/>
+      <c r="J42" s="37"/>
+      <c r="K42" s="37"/>
+      <c r="L42" s="37"/>
+      <c r="M42" s="37"/>
+      <c r="N42" s="37"/>
+      <c r="O42" s="37"/>
+      <c r="P42" s="37"/>
+      <c r="Q42" s="37"/>
+      <c r="R42" s="37"/>
+      <c r="S42" s="37"/>
+      <c r="T42" s="37"/>
+    </row>
+    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="28"/>
+      <c r="C43" s="36">
         <v>23</v>
       </c>
-      <c r="D43" s="44"/>
-      <c r="E43" s="44"/>
-      <c r="F43" s="44"/>
-      <c r="G43" s="44"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="44"/>
-      <c r="J43" s="44"/>
-      <c r="K43" s="44"/>
-      <c r="L43" s="44"/>
-      <c r="M43" s="44"/>
-      <c r="N43" s="44"/>
-      <c r="O43" s="44"/>
-      <c r="P43" s="44"/>
-      <c r="Q43" s="44"/>
-      <c r="R43" s="44"/>
-      <c r="S43" s="44"/>
-      <c r="T43" s="44"/>
-    </row>
-    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="35"/>
-      <c r="C44" s="43">
+      <c r="D43" s="37"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="37"/>
+      <c r="G43" s="37"/>
+      <c r="H43" s="37"/>
+      <c r="I43" s="37"/>
+      <c r="J43" s="37"/>
+      <c r="K43" s="37"/>
+      <c r="L43" s="37"/>
+      <c r="M43" s="37"/>
+      <c r="N43" s="37"/>
+      <c r="O43" s="37"/>
+      <c r="P43" s="37"/>
+      <c r="Q43" s="37"/>
+      <c r="R43" s="37"/>
+      <c r="S43" s="37"/>
+      <c r="T43" s="37"/>
+    </row>
+    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="28"/>
+      <c r="C44" s="36">
         <v>24</v>
       </c>
-      <c r="D44" s="44"/>
-      <c r="E44" s="44"/>
-      <c r="F44" s="44"/>
-      <c r="G44" s="44"/>
-      <c r="H44" s="44"/>
-      <c r="I44" s="44"/>
-      <c r="J44" s="44"/>
-      <c r="K44" s="44"/>
-      <c r="L44" s="44"/>
-      <c r="M44" s="44"/>
-      <c r="N44" s="44"/>
-      <c r="O44" s="44"/>
-      <c r="P44" s="44"/>
-      <c r="Q44" s="44"/>
-      <c r="R44" s="44"/>
-      <c r="S44" s="44"/>
-      <c r="T44" s="44"/>
-    </row>
-    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="35"/>
-      <c r="C45" s="43">
+      <c r="D44" s="37"/>
+      <c r="E44" s="37"/>
+      <c r="F44" s="37"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="37"/>
+      <c r="I44" s="37"/>
+      <c r="J44" s="37"/>
+      <c r="K44" s="37"/>
+      <c r="L44" s="37"/>
+      <c r="M44" s="37"/>
+      <c r="N44" s="37"/>
+      <c r="O44" s="37"/>
+      <c r="P44" s="37"/>
+      <c r="Q44" s="37"/>
+      <c r="R44" s="37"/>
+      <c r="S44" s="37"/>
+      <c r="T44" s="37"/>
+    </row>
+    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="28"/>
+      <c r="C45" s="36">
         <v>25</v>
       </c>
-      <c r="D45" s="44"/>
-      <c r="E45" s="44"/>
-      <c r="F45" s="44"/>
-      <c r="G45" s="44"/>
-      <c r="H45" s="44"/>
-      <c r="I45" s="44"/>
-      <c r="J45" s="44"/>
-      <c r="K45" s="44"/>
-      <c r="L45" s="44"/>
-      <c r="M45" s="44"/>
-      <c r="N45" s="44"/>
-      <c r="O45" s="44"/>
-      <c r="P45" s="44"/>
-      <c r="Q45" s="44"/>
-      <c r="R45" s="44"/>
-      <c r="S45" s="44"/>
-      <c r="T45" s="44"/>
-    </row>
-    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="35"/>
-      <c r="C46" s="43">
+      <c r="D45" s="37"/>
+      <c r="E45" s="37"/>
+      <c r="F45" s="37"/>
+      <c r="G45" s="37"/>
+      <c r="H45" s="37"/>
+      <c r="I45" s="37"/>
+      <c r="J45" s="37"/>
+      <c r="K45" s="37"/>
+      <c r="L45" s="37"/>
+      <c r="M45" s="37"/>
+      <c r="N45" s="37"/>
+      <c r="O45" s="37"/>
+      <c r="P45" s="37"/>
+      <c r="Q45" s="37"/>
+      <c r="R45" s="37"/>
+      <c r="S45" s="37"/>
+      <c r="T45" s="37"/>
+    </row>
+    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="28"/>
+      <c r="C46" s="36">
         <v>26</v>
       </c>
-      <c r="D46" s="44"/>
-      <c r="E46" s="44"/>
-      <c r="F46" s="44"/>
-      <c r="G46" s="44"/>
-      <c r="H46" s="44"/>
-      <c r="I46" s="44"/>
-      <c r="J46" s="44"/>
-      <c r="K46" s="44"/>
-      <c r="L46" s="44"/>
-      <c r="M46" s="44"/>
-      <c r="N46" s="44"/>
-      <c r="O46" s="44"/>
-      <c r="P46" s="44"/>
-      <c r="Q46" s="44"/>
-      <c r="R46" s="44"/>
-      <c r="S46" s="44"/>
-      <c r="T46" s="44"/>
-    </row>
-    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="35"/>
-      <c r="C47" s="43">
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="37"/>
+      <c r="I46" s="37"/>
+      <c r="J46" s="37"/>
+      <c r="K46" s="37"/>
+      <c r="L46" s="37"/>
+      <c r="M46" s="37"/>
+      <c r="N46" s="37"/>
+      <c r="O46" s="37"/>
+      <c r="P46" s="37"/>
+      <c r="Q46" s="37"/>
+      <c r="R46" s="37"/>
+      <c r="S46" s="37"/>
+      <c r="T46" s="37"/>
+    </row>
+    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="28"/>
+      <c r="C47" s="36">
         <v>27</v>
       </c>
-      <c r="D47" s="44"/>
-      <c r="E47" s="44"/>
-      <c r="F47" s="44"/>
-      <c r="G47" s="44"/>
-      <c r="H47" s="44"/>
-      <c r="I47" s="44"/>
-      <c r="J47" s="44"/>
-      <c r="K47" s="44"/>
-      <c r="L47" s="44"/>
-      <c r="M47" s="44"/>
-      <c r="N47" s="44"/>
-      <c r="O47" s="44"/>
-      <c r="P47" s="44"/>
-      <c r="Q47" s="44"/>
-      <c r="R47" s="44"/>
-      <c r="S47" s="44"/>
-      <c r="T47" s="44"/>
-    </row>
-    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="35"/>
-      <c r="C48" s="43">
+      <c r="D47" s="37"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="37"/>
+      <c r="I47" s="37"/>
+      <c r="J47" s="37"/>
+      <c r="K47" s="37"/>
+      <c r="L47" s="37"/>
+      <c r="M47" s="37"/>
+      <c r="N47" s="37"/>
+      <c r="O47" s="37"/>
+      <c r="P47" s="37"/>
+      <c r="Q47" s="37"/>
+      <c r="R47" s="37"/>
+      <c r="S47" s="37"/>
+      <c r="T47" s="37"/>
+    </row>
+    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="28"/>
+      <c r="C48" s="36">
         <v>28</v>
       </c>
-      <c r="D48" s="44"/>
-      <c r="E48" s="44"/>
-      <c r="F48" s="44"/>
-      <c r="G48" s="44"/>
-      <c r="H48" s="44"/>
-      <c r="I48" s="44"/>
-      <c r="J48" s="44"/>
-      <c r="K48" s="44"/>
-      <c r="L48" s="44"/>
-      <c r="M48" s="44"/>
-      <c r="N48" s="44"/>
-      <c r="O48" s="44"/>
-      <c r="P48" s="44"/>
-      <c r="Q48" s="44"/>
-      <c r="R48" s="44"/>
-      <c r="S48" s="44"/>
-      <c r="T48" s="44"/>
-    </row>
-    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="35"/>
-      <c r="C49" s="43">
+      <c r="D48" s="37"/>
+      <c r="E48" s="37"/>
+      <c r="F48" s="37"/>
+      <c r="G48" s="37"/>
+      <c r="H48" s="37"/>
+      <c r="I48" s="37"/>
+      <c r="J48" s="37"/>
+      <c r="K48" s="37"/>
+      <c r="L48" s="37"/>
+      <c r="M48" s="37"/>
+      <c r="N48" s="37"/>
+      <c r="O48" s="37"/>
+      <c r="P48" s="37"/>
+      <c r="Q48" s="37"/>
+      <c r="R48" s="37"/>
+      <c r="S48" s="37"/>
+      <c r="T48" s="37"/>
+    </row>
+    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="28"/>
+      <c r="C49" s="36">
         <v>29</v>
       </c>
-      <c r="D49" s="44"/>
-      <c r="E49" s="44"/>
-      <c r="F49" s="44"/>
-      <c r="G49" s="44"/>
-      <c r="H49" s="44"/>
-      <c r="I49" s="44"/>
-      <c r="J49" s="44"/>
-      <c r="K49" s="44"/>
-      <c r="L49" s="44"/>
-      <c r="M49" s="44"/>
-      <c r="N49" s="44"/>
-      <c r="O49" s="44"/>
-      <c r="P49" s="44"/>
-      <c r="Q49" s="44"/>
-      <c r="R49" s="44"/>
-      <c r="S49" s="44"/>
-      <c r="T49" s="44"/>
-    </row>
-    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="35"/>
-      <c r="C50" s="43">
+      <c r="D49" s="37"/>
+      <c r="E49" s="37"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="37"/>
+      <c r="H49" s="37"/>
+      <c r="I49" s="37"/>
+      <c r="J49" s="37"/>
+      <c r="K49" s="37"/>
+      <c r="L49" s="37"/>
+      <c r="M49" s="37"/>
+      <c r="N49" s="37"/>
+      <c r="O49" s="37"/>
+      <c r="P49" s="37"/>
+      <c r="Q49" s="37"/>
+      <c r="R49" s="37"/>
+      <c r="S49" s="37"/>
+      <c r="T49" s="37"/>
+    </row>
+    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="28"/>
+      <c r="C50" s="36">
         <v>30</v>
       </c>
-      <c r="D50" s="44"/>
-      <c r="E50" s="44"/>
-      <c r="F50" s="44"/>
-      <c r="G50" s="44"/>
-      <c r="H50" s="44"/>
-      <c r="I50" s="44"/>
-      <c r="J50" s="44"/>
-      <c r="K50" s="44"/>
-      <c r="L50" s="44"/>
-      <c r="M50" s="44"/>
-      <c r="N50" s="44"/>
-      <c r="O50" s="44"/>
-      <c r="P50" s="44"/>
-      <c r="Q50" s="44"/>
-      <c r="R50" s="44"/>
-      <c r="S50" s="44"/>
-      <c r="T50" s="44"/>
-    </row>
-    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="35"/>
-      <c r="C51" s="43">
+      <c r="D50" s="37"/>
+      <c r="E50" s="37"/>
+      <c r="F50" s="37"/>
+      <c r="G50" s="37"/>
+      <c r="H50" s="37"/>
+      <c r="I50" s="37"/>
+      <c r="J50" s="37"/>
+      <c r="K50" s="37"/>
+      <c r="L50" s="37"/>
+      <c r="M50" s="37"/>
+      <c r="N50" s="37"/>
+      <c r="O50" s="37"/>
+      <c r="P50" s="37"/>
+      <c r="Q50" s="37"/>
+      <c r="R50" s="37"/>
+      <c r="S50" s="37"/>
+      <c r="T50" s="37"/>
+    </row>
+    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="28"/>
+      <c r="C51" s="36">
         <v>31</v>
       </c>
-      <c r="D51" s="44"/>
-      <c r="E51" s="44"/>
-      <c r="F51" s="44"/>
-      <c r="G51" s="44"/>
-      <c r="H51" s="44"/>
-      <c r="I51" s="44"/>
-      <c r="J51" s="44"/>
-      <c r="K51" s="44"/>
-      <c r="L51" s="44"/>
-      <c r="M51" s="44"/>
-      <c r="N51" s="44"/>
-      <c r="O51" s="44"/>
-      <c r="P51" s="44"/>
-      <c r="Q51" s="44"/>
-      <c r="R51" s="44"/>
-      <c r="S51" s="44"/>
-      <c r="T51" s="44"/>
+      <c r="D51" s="37"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="37"/>
+      <c r="G51" s="37"/>
+      <c r="H51" s="37"/>
+      <c r="I51" s="37"/>
+      <c r="J51" s="37"/>
+      <c r="K51" s="37"/>
+      <c r="L51" s="37"/>
+      <c r="M51" s="37"/>
+      <c r="N51" s="37"/>
+      <c r="O51" s="37"/>
+      <c r="P51" s="37"/>
+      <c r="Q51" s="37"/>
+      <c r="R51" s="37"/>
+      <c r="S51" s="37"/>
+      <c r="T51" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="T19:T20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="Q19:Q20"/>
-    <mergeCell ref="R19:R20"/>
-    <mergeCell ref="S19:S20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="D6:J6"/>
     <mergeCell ref="C11:T11"/>
     <mergeCell ref="E13:K13"/>
     <mergeCell ref="E14:K14"/>
@@ -2466,9 +2453,22 @@
     <mergeCell ref="L18:P18"/>
     <mergeCell ref="Q17:S18"/>
     <mergeCell ref="T17:T18"/>
-    <mergeCell ref="B3:T3"/>
-    <mergeCell ref="D5:J5"/>
-    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="T19:T20"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="Q19:Q20"/>
+    <mergeCell ref="R19:R20"/>
+    <mergeCell ref="S19:S20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2477,31 +2477,31 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F6E3FC4-92B9-4B14-9A38-1F80DD1D104A}">
   <dimension ref="B2:U51"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="6.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="6.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="36" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="32" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="33.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="31.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="20.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="33.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.33203125" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" ht="24" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2523,31 +2523,31 @@
       <c r="T2" s="4"/>
       <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="2:21" ht="24" x14ac:dyDescent="0.4">
-      <c r="B3" s="28" t="s">
+    <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B3" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="29"/>
-      <c r="R3" s="29"/>
-      <c r="S3" s="29"/>
-      <c r="T3" s="30"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="55"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -2568,18 +2568,18 @@
       <c r="S4" s="7"/>
       <c r="T4" s="8"/>
     </row>
-    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6"/>
       <c r="C5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -2591,18 +2591,18 @@
       <c r="S5" s="18"/>
       <c r="T5" s="19"/>
     </row>
-    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
       <c r="C6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="57"/>
+      <c r="J6" s="57"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
@@ -2614,7 +2614,7 @@
       <c r="S6" s="18"/>
       <c r="T6" s="19"/>
     </row>
-    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6"/>
       <c r="C7" s="18"/>
       <c r="D7" s="20"/>
@@ -2635,7 +2635,7 @@
       <c r="S7" s="18"/>
       <c r="T7" s="19"/>
     </row>
-    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6"/>
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
@@ -2656,34 +2656,34 @@
       <c r="S8" s="18"/>
       <c r="T8" s="19"/>
     </row>
-    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="16"/>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32" t="s">
+      <c r="D9" s="58"/>
+      <c r="E9" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59"/>
       <c r="J9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="32" t="s">
+      <c r="K9" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="32"/>
-      <c r="M9" s="32"/>
-      <c r="N9" s="32"/>
-      <c r="O9" s="32"/>
-      <c r="P9" s="31" t="s">
+      <c r="L9" s="59"/>
+      <c r="M9" s="59"/>
+      <c r="N9" s="59"/>
+      <c r="O9" s="59"/>
+      <c r="P9" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="Q9" s="31"/>
-      <c r="R9" s="31"/>
+      <c r="Q9" s="58"/>
+      <c r="R9" s="58"/>
       <c r="S9" s="22" t="s">
         <v>24</v>
       </c>
@@ -2691,7 +2691,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>7</v>
       </c>
@@ -2746,7 +2746,7 @@
       <c r="S10" s="25"/>
       <c r="T10" s="26"/>
     </row>
-    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="9">
         <v>1</v>
       </c>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="T11" s="11"/>
     </row>
-    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>2</v>
       </c>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="T12" s="11"/>
     </row>
-    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
         <v>3</v>
       </c>
@@ -2907,7 +2907,7 @@
       </c>
       <c r="T13" s="11"/>
     </row>
-    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="9">
         <v>4</v>
       </c>
@@ -2954,7 +2954,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="11"/>
     </row>
-    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="9">
         <v>5</v>
       </c>
@@ -2999,7 +2999,7 @@
       <c r="S15" s="10"/>
       <c r="T15" s="11"/>
     </row>
-    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="9">
         <v>6</v>
       </c>
@@ -3042,7 +3042,7 @@
       <c r="S16" s="10"/>
       <c r="T16" s="11"/>
     </row>
-    <row r="17" spans="2:20" ht="70.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="9">
         <v>7</v>
       </c>
@@ -3071,16 +3071,16 @@
         <v>56</v>
       </c>
       <c r="K17" s="10">
-        <v>0.56399999999999995</v>
+        <v>0.59599999999999997</v>
       </c>
       <c r="L17" s="10">
-        <v>0.56499999999999995</v>
+        <v>0.59899999999999998</v>
       </c>
       <c r="M17" s="10">
-        <v>0.56399999999999995</v>
+        <v>0.59599999999999997</v>
       </c>
       <c r="N17" s="10">
-        <v>0.56299999999999994</v>
+        <v>0.59699999999999998</v>
       </c>
       <c r="O17" s="10"/>
       <c r="P17" s="10"/>
@@ -3089,7 +3089,7 @@
       <c r="S17" s="10"/>
       <c r="T17" s="11"/>
     </row>
-    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9">
         <v>8</v>
       </c>
@@ -3136,7 +3136,7 @@
       <c r="S18" s="10"/>
       <c r="T18" s="11"/>
     </row>
-    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>9</v>
       </c>
@@ -3159,7 +3159,7 @@
       <c r="S19" s="10"/>
       <c r="T19" s="11"/>
     </row>
-    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="9">
         <v>10</v>
       </c>
@@ -3182,7 +3182,7 @@
       <c r="S20" s="10"/>
       <c r="T20" s="11"/>
     </row>
-    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9">
         <v>11</v>
       </c>
@@ -3205,7 +3205,7 @@
       <c r="S21" s="10"/>
       <c r="T21" s="11"/>
     </row>
-    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
         <v>12</v>
       </c>
@@ -3228,7 +3228,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="11"/>
     </row>
-    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
@@ -3251,7 +3251,7 @@
       <c r="S23" s="10"/>
       <c r="T23" s="11"/>
     </row>
-    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9">
         <v>14</v>
       </c>
@@ -3274,7 +3274,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="11"/>
     </row>
-    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9">
         <v>15</v>
       </c>
@@ -3297,7 +3297,7 @@
       <c r="S25" s="10"/>
       <c r="T25" s="11"/>
     </row>
-    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
         <v>16</v>
       </c>
@@ -3320,7 +3320,7 @@
       <c r="S26" s="10"/>
       <c r="T26" s="11"/>
     </row>
-    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="9">
         <v>17</v>
       </c>
@@ -3343,7 +3343,7 @@
       <c r="S27" s="10"/>
       <c r="T27" s="11"/>
     </row>
-    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="9">
         <v>18</v>
       </c>
@@ -3366,7 +3366,7 @@
       <c r="S28" s="10"/>
       <c r="T28" s="11"/>
     </row>
-    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="9">
         <v>19</v>
       </c>
@@ -3389,7 +3389,7 @@
       <c r="S29" s="10"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="9">
         <v>20</v>
       </c>
@@ -3412,7 +3412,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="11"/>
     </row>
-    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="9">
         <v>21</v>
       </c>
@@ -3435,7 +3435,7 @@
       <c r="S31" s="10"/>
       <c r="T31" s="11"/>
     </row>
-    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9">
         <v>22</v>
       </c>
@@ -3458,7 +3458,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="11"/>
     </row>
-    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="9">
         <v>23</v>
       </c>
@@ -3481,7 +3481,7 @@
       <c r="S33" s="10"/>
       <c r="T33" s="11"/>
     </row>
-    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="9">
         <v>24</v>
       </c>
@@ -3504,7 +3504,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="11"/>
     </row>
-    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="9">
         <v>25</v>
       </c>
@@ -3527,7 +3527,7 @@
       <c r="S35" s="10"/>
       <c r="T35" s="11"/>
     </row>
-    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9">
         <v>26</v>
       </c>
@@ -3550,7 +3550,7 @@
       <c r="S36" s="10"/>
       <c r="T36" s="11"/>
     </row>
-    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="9">
         <v>27</v>
       </c>
@@ -3573,7 +3573,7 @@
       <c r="S37" s="10"/>
       <c r="T37" s="11"/>
     </row>
-    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="9">
         <v>28</v>
       </c>
@@ -3596,7 +3596,7 @@
       <c r="S38" s="10"/>
       <c r="T38" s="11"/>
     </row>
-    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
         <v>29</v>
       </c>
@@ -3619,7 +3619,7 @@
       <c r="S39" s="10"/>
       <c r="T39" s="11"/>
     </row>
-    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9">
         <v>30</v>
       </c>
@@ -3642,7 +3642,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="11"/>
     </row>
-    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="9">
         <v>31</v>
       </c>
@@ -3665,7 +3665,7 @@
       <c r="S41" s="10"/>
       <c r="T41" s="11"/>
     </row>
-    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="9">
         <v>32</v>
       </c>
@@ -3688,7 +3688,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="11"/>
     </row>
-    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="9">
         <v>33</v>
       </c>
@@ -3711,7 +3711,7 @@
       <c r="S43" s="10"/>
       <c r="T43" s="11"/>
     </row>
-    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="9">
         <v>34</v>
       </c>
@@ -3734,7 +3734,7 @@
       <c r="S44" s="10"/>
       <c r="T44" s="11"/>
     </row>
-    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="9">
         <v>35</v>
       </c>
@@ -3757,7 +3757,7 @@
       <c r="S45" s="10"/>
       <c r="T45" s="11"/>
     </row>
-    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="9">
         <v>36</v>
       </c>
@@ -3780,7 +3780,7 @@
       <c r="S46" s="10"/>
       <c r="T46" s="11"/>
     </row>
-    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="9">
         <v>37</v>
       </c>
@@ -3803,7 +3803,7 @@
       <c r="S47" s="10"/>
       <c r="T47" s="11"/>
     </row>
-    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="9">
         <v>38</v>
       </c>
@@ -3826,7 +3826,7 @@
       <c r="S48" s="10"/>
       <c r="T48" s="11"/>
     </row>
-    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="9">
         <v>39</v>
       </c>
@@ -3849,7 +3849,7 @@
       <c r="S49" s="10"/>
       <c r="T49" s="11"/>
     </row>
-    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12">
         <v>40</v>
       </c>
@@ -3872,7 +3872,7 @@
       <c r="S50" s="13"/>
       <c r="T50" s="14"/>
     </row>
-    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C51" s="15" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Add model notes for the Keras models
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\git-school\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6908FD49-62B1-41E8-ADA7-3AA057B8B31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C3C785B-3D61-48A8-B3D7-8BB8F846ABE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
   <sheets>
     <sheet name="Model Iteration Log Filip" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="88">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -283,6 +283,42 @@
   </si>
   <si>
     <t>Sentence_Tok', "bert_embedding"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relatively quick to run. Requires more resources compared to a Sklearn model, but less compared to an LSTM model or Transformer-based models. </t>
+  </si>
+  <si>
+    <t>Can't fully understand the linguistic patterns in the training data required for distinguishing between the 7 classes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still relatively quick to run. It requires a bit more resources compared to the SimpleRNN-v0 model, which only had one recurrent layer, but it is still less computationally expensive compared to future models. </t>
+  </si>
+  <si>
+    <t>While somewhat better than the SimpleRNN-v0 model, it still can't fully understand the linguistic patterns in the training data required for distinguishing between the 7 classes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The LSTM layer is much better at understanding the linguistic patterns in the training data compared to the SimpleRNN layer or the Sklearn models. Its memory gates make it much more efficient at modelling the data. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires more computational power than the previously logged models. It takes more time to run. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The two LSTM layers improve the performance over the LSTM-v0 model. The model has a good modelling capability, being the first one so far to surpass the criteria for the F1 score. </t>
+  </si>
+  <si>
+    <t>Requires more computational power than the previously logged models. It takes more time to run.</t>
+  </si>
+  <si>
+    <t>Uses the same architecture as the best-performing base model: LSTM-v1, but we added additional features as inputs, which slightly increased the model's performance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The added features make it require more computational power to run. The training time also slightly increases with the addition of these features. </t>
+  </si>
+  <si>
+    <t>We believe that stacking these features might have introduced confusion for the model.</t>
+  </si>
+  <si>
+    <t>Uses the same architecture as the best-performing base model: LSTM-v1. To address our concern with the previous model, we only added one feature: the BERT embeddings. This proved our assumption correct, as the results saw a slight increase compared to the last model. It also requires less computational power to run compared to the LSTM-v2 model</t>
   </si>
 </sst>
 </file>
@@ -706,64 +742,64 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1154,27 +1190,27 @@
       <c r="U2" s="5"/>
     </row>
     <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="51"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="38"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="39"/>
       <c r="U3" s="5"/>
     </row>
     <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -1203,13 +1239,13 @@
       <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
@@ -1226,13 +1262,13 @@
       <c r="C6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
@@ -1330,26 +1366,26 @@
     </row>
     <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="27"/>
-      <c r="C11" s="54" t="s">
+      <c r="C11" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="55"/>
-      <c r="E11" s="55"/>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="55"/>
-      <c r="J11" s="55"/>
-      <c r="K11" s="55"/>
-      <c r="L11" s="55"/>
-      <c r="M11" s="55"/>
-      <c r="N11" s="55"/>
-      <c r="O11" s="55"/>
-      <c r="P11" s="55"/>
-      <c r="Q11" s="55"/>
-      <c r="R11" s="55"/>
-      <c r="S11" s="55"/>
-      <c r="T11" s="55"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
+      <c r="Q11" s="43"/>
+      <c r="R11" s="43"/>
+      <c r="S11" s="43"/>
+      <c r="T11" s="43"/>
     </row>
     <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="27"/>
@@ -1378,13 +1414,13 @@
       <c r="D13" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="56"/>
-      <c r="F13" s="56"/>
-      <c r="G13" s="56"/>
-      <c r="H13" s="56"/>
-      <c r="I13" s="56"/>
-      <c r="J13" s="56"/>
-      <c r="K13" s="56"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
       <c r="L13" s="32"/>
       <c r="M13" s="32"/>
       <c r="N13" s="32"/>
@@ -1401,13 +1437,13 @@
       <c r="D14" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="47"/>
-      <c r="J14" s="47"/>
-      <c r="K14" s="47"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="45"/>
       <c r="L14" s="32"/>
       <c r="M14" s="32"/>
       <c r="N14" s="32"/>
@@ -1461,79 +1497,79 @@
       <c r="T16" s="32"/>
     </row>
     <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="43"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="41" t="s">
+      <c r="B17" s="46"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="41"/>
-      <c r="F17" s="39" t="s">
+      <c r="E17" s="49"/>
+      <c r="F17" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="41" t="s">
+      <c r="G17" s="51"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="L17" s="39" t="s">
+      <c r="L17" s="51" t="s">
         <v>55</v>
       </c>
-      <c r="M17" s="39"/>
-      <c r="N17" s="39"/>
-      <c r="O17" s="39"/>
-      <c r="P17" s="39"/>
-      <c r="Q17" s="41" t="s">
+      <c r="M17" s="51"/>
+      <c r="N17" s="51"/>
+      <c r="O17" s="51"/>
+      <c r="P17" s="51"/>
+      <c r="Q17" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="R17" s="41"/>
-      <c r="S17" s="41"/>
-      <c r="T17" s="39" t="s">
+      <c r="R17" s="49"/>
+      <c r="S17" s="49"/>
+      <c r="T17" s="51" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="43"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="38"/>
-      <c r="L18" s="40" t="s">
+      <c r="B18" s="46"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="52"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="52"/>
+      <c r="I18" s="52"/>
+      <c r="J18" s="52"/>
+      <c r="K18" s="50"/>
+      <c r="L18" s="56" t="s">
         <v>56</v>
       </c>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
-      <c r="O18" s="40"/>
-      <c r="P18" s="40"/>
-      <c r="Q18" s="38"/>
-      <c r="R18" s="38"/>
-      <c r="S18" s="38"/>
-      <c r="T18" s="42"/>
+      <c r="M18" s="56"/>
+      <c r="N18" s="56"/>
+      <c r="O18" s="56"/>
+      <c r="P18" s="56"/>
+      <c r="Q18" s="50"/>
+      <c r="R18" s="50"/>
+      <c r="S18" s="50"/>
+      <c r="T18" s="52"/>
     </row>
     <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="43"/>
-      <c r="C19" s="44" t="s">
+      <c r="B19" s="46"/>
+      <c r="C19" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="37" t="s">
+      <c r="E19" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="F19" s="46" t="s">
+      <c r="F19" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="G19" s="46" t="s">
+      <c r="G19" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="46" t="s">
+      <c r="H19" s="53" t="s">
         <v>14</v>
       </c>
       <c r="I19" s="33" t="s">
@@ -1542,61 +1578,61 @@
       <c r="J19" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="K19" s="37" t="s">
+      <c r="K19" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="L19" s="46" t="s">
+      <c r="L19" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="M19" s="46" t="s">
+      <c r="M19" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="N19" s="46" t="s">
+      <c r="N19" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="O19" s="46" t="s">
+      <c r="O19" s="53" t="s">
         <v>19</v>
       </c>
       <c r="P19" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="Q19" s="37" t="s">
+      <c r="Q19" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="R19" s="37" t="s">
+      <c r="R19" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="S19" s="37" t="s">
+      <c r="S19" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="T19" s="46"/>
+      <c r="T19" s="53"/>
     </row>
     <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="43"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
       <c r="I20" s="34" t="s">
         <v>58</v>
       </c>
       <c r="J20" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="K20" s="38"/>
-      <c r="L20" s="42"/>
-      <c r="M20" s="42"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="42"/>
+      <c r="K20" s="50"/>
+      <c r="L20" s="52"/>
+      <c r="M20" s="52"/>
+      <c r="N20" s="52"/>
+      <c r="O20" s="52"/>
       <c r="P20" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="Q20" s="38"/>
-      <c r="R20" s="38"/>
-      <c r="S20" s="38"/>
-      <c r="T20" s="42"/>
+      <c r="Q20" s="50"/>
+      <c r="R20" s="50"/>
+      <c r="S20" s="50"/>
+      <c r="T20" s="52"/>
     </row>
     <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="27"/>
@@ -2465,27 +2501,6 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B3:T3"/>
-    <mergeCell ref="D5:J5"/>
-    <mergeCell ref="D6:J6"/>
-    <mergeCell ref="C11:T11"/>
-    <mergeCell ref="E13:K13"/>
-    <mergeCell ref="E14:K14"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:E18"/>
-    <mergeCell ref="F17:J18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
     <mergeCell ref="S19:S20"/>
     <mergeCell ref="L17:P17"/>
     <mergeCell ref="L18:P18"/>
@@ -2496,6 +2511,27 @@
     <mergeCell ref="O19:O20"/>
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="E14:K14"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:E18"/>
+    <mergeCell ref="F17:J18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="C11:T11"/>
+    <mergeCell ref="E13:K13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2551,27 +2587,27 @@
       <c r="U2" s="5"/>
     </row>
     <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="51"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="38"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="39"/>
       <c r="U3" s="5"/>
     </row>
     <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -2600,13 +2636,13 @@
       <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
@@ -2623,13 +2659,13 @@
       <c r="C6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
@@ -3112,8 +3148,12 @@
         <v>0.55300000000000005</v>
       </c>
       <c r="O17" s="10"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="10"/>
+      <c r="P17" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q17" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="R17" s="10"/>
       <c r="S17" s="10"/>
       <c r="T17" s="11"/>
@@ -3159,13 +3199,17 @@
         <v>0.59699999999999998</v>
       </c>
       <c r="O18" s="10"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10"/>
+      <c r="P18" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q18" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="R18" s="10"/>
       <c r="S18" s="10"/>
       <c r="T18" s="11"/>
     </row>
-    <row r="19" spans="2:20" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:20" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>9</v>
       </c>
@@ -3206,8 +3250,12 @@
         <v>0.71299999999999997</v>
       </c>
       <c r="O19" s="10"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="10"/>
+      <c r="P19" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>81</v>
+      </c>
       <c r="R19" s="10"/>
       <c r="S19" s="10"/>
       <c r="T19" s="11"/>
@@ -3253,8 +3301,12 @@
         <v>0.76700000000000002</v>
       </c>
       <c r="O20" s="10"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="10"/>
+      <c r="P20" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q20" s="10" t="s">
+        <v>83</v>
+      </c>
       <c r="R20" s="10"/>
       <c r="S20" s="10"/>
       <c r="T20" s="11"/>
@@ -3300,13 +3352,19 @@
         <v>0.79300000000000004</v>
       </c>
       <c r="O21" s="10"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
+      <c r="P21" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q21" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="R21" s="10" t="s">
+        <v>86</v>
+      </c>
       <c r="S21" s="10"/>
       <c r="T21" s="11"/>
     </row>
-    <row r="22" spans="2:20" ht="80.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:20" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
         <v>12</v>
       </c>
@@ -3347,7 +3405,9 @@
         <v>0.79900000000000004</v>
       </c>
       <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
+      <c r="P22" s="10" t="s">
+        <v>87</v>
+      </c>
       <c r="Q22" s="10"/>
       <c r="R22" s="10"/>
       <c r="S22" s="10"/>

</xml_diff>

<commit_message>
Add trasnformer models stats
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\git-school\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C3C785B-3D61-48A8-B3D7-8BB8F846ABE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42CAFEE-C635-4AD6-AD2D-5AAD5CBE8437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
   <sheets>
     <sheet name="Model Iteration Log Filip" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="98">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -97,10 +97,6 @@
   </si>
   <si>
     <t>F1 score</t>
-  </si>
-  <si>
-    <t>Other metrics 
-(if applicable)</t>
   </si>
   <si>
     <t>Strenghts</t>
@@ -319,6 +315,39 @@
   </si>
   <si>
     <t>Uses the same architecture as the best-performing base model: LSTM-v1. To address our concern with the previous model, we only added one feature: the BERT embeddings. This proved our assumption correct, as the results saw a slight increase compared to the last model. It also requires less computational power to run compared to the LSTM-v2 model</t>
+  </si>
+  <si>
+    <t>Accuracy - Test Set</t>
+  </si>
+  <si>
+    <t>F1 score - Test Set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Its performance increase didn't justify the effort put into it. Even though we added features that we assumed would increase its performance, the difference in accuracy and weighted F1 score was not as big as we expected.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> We believe that the performance increase starting to plateau means that we have reached or almost reached the peak performance of the current architecture, meaning that we will now move on to more powerful models, namely, Transformer-based ones, like BERT or ROBERTA.</t>
+  </si>
+  <si>
+    <t>DistilBERT-base-uncased-sst-2-english</t>
+  </si>
+  <si>
+    <t>transformers</t>
+  </si>
+  <si>
+    <t>final_dataset.csv - 5000 samples per class</t>
+  </si>
+  <si>
+    <t>transformers.AutoTokenizer</t>
+  </si>
+  <si>
+    <t>Sentence_Tok</t>
+  </si>
+  <si>
+    <t>learning_rate=2e-5, per_device_train_batch_size=16, num_train_epochs=5, weight_decay=0.01, metric_for_best_model="accuracy",</t>
+  </si>
+  <si>
+    <t>BERT-base-uncased</t>
   </si>
 </sst>
 </file>
@@ -742,6 +771,42 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -764,42 +829,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1190,27 +1219,27 @@
       <c r="U2" s="5"/>
     </row>
     <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="38"/>
-      <c r="P3" s="38"/>
-      <c r="Q3" s="38"/>
-      <c r="R3" s="38"/>
-      <c r="S3" s="38"/>
-      <c r="T3" s="39"/>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="50"/>
+      <c r="L3" s="50"/>
+      <c r="M3" s="50"/>
+      <c r="N3" s="50"/>
+      <c r="O3" s="50"/>
+      <c r="P3" s="50"/>
+      <c r="Q3" s="50"/>
+      <c r="R3" s="50"/>
+      <c r="S3" s="50"/>
+      <c r="T3" s="51"/>
       <c r="U3" s="5"/>
     </row>
     <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -1239,13 +1268,13 @@
       <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="52"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
@@ -1262,13 +1291,13 @@
       <c r="C6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="53"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
@@ -1366,26 +1395,26 @@
     </row>
     <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="27"/>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-      <c r="O11" s="43"/>
-      <c r="P11" s="43"/>
-      <c r="Q11" s="43"/>
-      <c r="R11" s="43"/>
-      <c r="S11" s="43"/>
-      <c r="T11" s="43"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="55"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
+      <c r="J11" s="55"/>
+      <c r="K11" s="55"/>
+      <c r="L11" s="55"/>
+      <c r="M11" s="55"/>
+      <c r="N11" s="55"/>
+      <c r="O11" s="55"/>
+      <c r="P11" s="55"/>
+      <c r="Q11" s="55"/>
+      <c r="R11" s="55"/>
+      <c r="S11" s="55"/>
+      <c r="T11" s="55"/>
     </row>
     <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="27"/>
@@ -1414,13 +1443,13 @@
       <c r="D13" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="44"/>
-      <c r="J13" s="44"/>
-      <c r="K13" s="44"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="56"/>
+      <c r="G13" s="56"/>
+      <c r="H13" s="56"/>
+      <c r="I13" s="56"/>
+      <c r="J13" s="56"/>
+      <c r="K13" s="56"/>
       <c r="L13" s="32"/>
       <c r="M13" s="32"/>
       <c r="N13" s="32"/>
@@ -1437,13 +1466,13 @@
       <c r="D14" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="45"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
       <c r="L14" s="32"/>
       <c r="M14" s="32"/>
       <c r="N14" s="32"/>
@@ -1497,142 +1526,142 @@
       <c r="T16" s="32"/>
     </row>
     <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="46"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="49" t="s">
+      <c r="B17" s="44"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="49"/>
-      <c r="F17" s="51" t="s">
+      <c r="E17" s="41"/>
+      <c r="F17" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="G17" s="51"/>
-      <c r="H17" s="51"/>
-      <c r="I17" s="51"/>
-      <c r="J17" s="51"/>
-      <c r="K17" s="49" t="s">
+      <c r="G17" s="39"/>
+      <c r="H17" s="39"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="39"/>
+      <c r="K17" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="L17" s="51" t="s">
+      <c r="L17" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="M17" s="39"/>
+      <c r="N17" s="39"/>
+      <c r="O17" s="39"/>
+      <c r="P17" s="39"/>
+      <c r="Q17" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="R17" s="41"/>
+      <c r="S17" s="41"/>
+      <c r="T17" s="39" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="44"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="38"/>
+      <c r="L18" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="M17" s="51"/>
-      <c r="N17" s="51"/>
-      <c r="O17" s="51"/>
-      <c r="P17" s="51"/>
-      <c r="Q17" s="49" t="s">
-        <v>6</v>
-      </c>
-      <c r="R17" s="49"/>
-      <c r="S17" s="49"/>
-      <c r="T17" s="51" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="46"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="52"/>
-      <c r="G18" s="52"/>
-      <c r="H18" s="52"/>
-      <c r="I18" s="52"/>
-      <c r="J18" s="52"/>
-      <c r="K18" s="50"/>
-      <c r="L18" s="56" t="s">
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
+      <c r="O18" s="40"/>
+      <c r="P18" s="40"/>
+      <c r="Q18" s="38"/>
+      <c r="R18" s="38"/>
+      <c r="S18" s="38"/>
+      <c r="T18" s="42"/>
+    </row>
+    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="44"/>
+      <c r="C19" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="43" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="I19" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="M18" s="56"/>
-      <c r="N18" s="56"/>
-      <c r="O18" s="56"/>
-      <c r="P18" s="56"/>
-      <c r="Q18" s="50"/>
-      <c r="R18" s="50"/>
-      <c r="S18" s="50"/>
-      <c r="T18" s="52"/>
-    </row>
-    <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="46"/>
-      <c r="C19" s="55" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="54" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="53" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="53" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="53" t="s">
-        <v>14</v>
-      </c>
-      <c r="I19" s="33" t="s">
+      <c r="J19" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="K19" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="L19" s="43" t="s">
+        <v>16</v>
+      </c>
+      <c r="M19" s="43" t="s">
+        <v>17</v>
+      </c>
+      <c r="N19" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="O19" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="P19" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q19" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="R19" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="S19" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="T19" s="43"/>
+    </row>
+    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="44"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="J19" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="K19" s="54" t="s">
-        <v>15</v>
-      </c>
-      <c r="L19" s="53" t="s">
-        <v>16</v>
-      </c>
-      <c r="M19" s="53" t="s">
-        <v>17</v>
-      </c>
-      <c r="N19" s="53" t="s">
-        <v>18</v>
-      </c>
-      <c r="O19" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="P19" s="33" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q19" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="R19" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="S19" s="54" t="s">
-        <v>22</v>
-      </c>
-      <c r="T19" s="53"/>
-    </row>
-    <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="46"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="50"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="34" t="s">
-        <v>58</v>
-      </c>
       <c r="J20" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="K20" s="50"/>
-      <c r="L20" s="52"/>
-      <c r="M20" s="52"/>
-      <c r="N20" s="52"/>
-      <c r="O20" s="52"/>
+        <v>57</v>
+      </c>
+      <c r="K20" s="38"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="42"/>
+      <c r="N20" s="42"/>
+      <c r="O20" s="42"/>
       <c r="P20" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q20" s="50"/>
-      <c r="R20" s="50"/>
-      <c r="S20" s="50"/>
-      <c r="T20" s="52"/>
+        <v>57</v>
+      </c>
+      <c r="Q20" s="38"/>
+      <c r="R20" s="38"/>
+      <c r="S20" s="38"/>
+      <c r="T20" s="42"/>
     </row>
     <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="27"/>
@@ -1640,26 +1669,26 @@
         <v>1</v>
       </c>
       <c r="D21" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="36" t="s">
+      <c r="F21" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="36" t="s">
+      <c r="G21" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G21" s="36" t="s">
+      <c r="H21" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="H21" s="36" t="s">
+      <c r="I21" s="36" t="s">
         <v>32</v>
-      </c>
-      <c r="I21" s="36" t="s">
-        <v>33</v>
       </c>
       <c r="J21" s="36"/>
       <c r="K21" s="36" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L21" s="36">
         <v>0.24399999999999999</v>
@@ -1675,16 +1704,16 @@
       </c>
       <c r="P21" s="36"/>
       <c r="Q21" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="R21" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="R21" s="36" t="s">
+      <c r="S21" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="S21" s="36" t="s">
+      <c r="T21" s="36" t="s">
         <v>37</v>
-      </c>
-      <c r="T21" s="36" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="22" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1693,26 +1722,26 @@
         <v>2</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E22" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F22" s="36" t="s">
+      <c r="G22" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G22" s="36" t="s">
+      <c r="H22" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="36" t="s">
+      <c r="I22" s="36" t="s">
         <v>32</v>
-      </c>
-      <c r="I22" s="36" t="s">
-        <v>33</v>
       </c>
       <c r="J22" s="36"/>
       <c r="K22" s="36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L22" s="36">
         <v>0.29299999999999998</v>
@@ -1728,12 +1757,12 @@
       </c>
       <c r="P22" s="36"/>
       <c r="Q22" s="36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R22" s="36"/>
       <c r="S22" s="36"/>
       <c r="T22" s="36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1742,26 +1771,26 @@
         <v>3</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E23" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="36" t="s">
+      <c r="G23" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G23" s="36" t="s">
+      <c r="H23" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="H23" s="36" t="s">
+      <c r="I23" s="36" t="s">
         <v>32</v>
-      </c>
-      <c r="I23" s="36" t="s">
-        <v>33</v>
       </c>
       <c r="J23" s="36"/>
       <c r="K23" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L23" s="36">
         <v>0.252</v>
@@ -1777,16 +1806,16 @@
       </c>
       <c r="P23" s="36"/>
       <c r="Q23" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="R23" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="R23" s="36" t="s">
+      <c r="S23" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="S23" s="36" t="s">
-        <v>45</v>
-      </c>
       <c r="T23" s="36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1795,26 +1824,26 @@
         <v>4</v>
       </c>
       <c r="D24" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="36" t="s">
+      <c r="F24" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F24" s="36" t="s">
+      <c r="G24" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G24" s="36" t="s">
+      <c r="H24" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="H24" s="36" t="s">
-        <v>32</v>
-      </c>
       <c r="I24" s="36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J24" s="36"/>
       <c r="K24" s="36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L24" s="36">
         <v>0.248</v>
@@ -1840,26 +1869,26 @@
         <v>5</v>
       </c>
       <c r="D25" s="36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E25" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F25" s="36" t="s">
+      <c r="G25" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G25" s="36" t="s">
+      <c r="H25" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="H25" s="36" t="s">
-        <v>32</v>
-      </c>
       <c r="I25" s="36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J25" s="36"/>
       <c r="K25" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L25" s="36">
         <v>0.28699999999999998</v>
@@ -1885,26 +1914,26 @@
         <v>6</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E26" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F26" s="36" t="s">
+      <c r="G26" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G26" s="36" t="s">
+      <c r="H26" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="H26" s="36" t="s">
-        <v>32</v>
-      </c>
       <c r="I26" s="36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J26" s="36"/>
       <c r="K26" s="36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L26" s="36">
         <v>0.26200000000000001</v>
@@ -2501,6 +2530,27 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="C11:T11"/>
+    <mergeCell ref="E13:K13"/>
+    <mergeCell ref="E14:K14"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:E18"/>
+    <mergeCell ref="F17:J18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
     <mergeCell ref="S19:S20"/>
     <mergeCell ref="L17:P17"/>
     <mergeCell ref="L18:P18"/>
@@ -2511,27 +2561,6 @@
     <mergeCell ref="O19:O20"/>
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="E14:K14"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:E18"/>
-    <mergeCell ref="F17:J18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="B3:T3"/>
-    <mergeCell ref="D5:J5"/>
-    <mergeCell ref="D6:J6"/>
-    <mergeCell ref="C11:T11"/>
-    <mergeCell ref="E13:K13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2539,7 +2568,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F6E3FC4-92B9-4B14-9A38-1F80DD1D104A}">
-  <dimension ref="B2:U52"/>
+  <dimension ref="B2:V52"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="6.44140625" style="1" customWidth="1"/>
@@ -2555,16 +2584,17 @@
     <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
     <col min="13" max="13" width="14.33203125" style="1" customWidth="1"/>
     <col min="14" max="14" width="15.109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.44140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="33.109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.5546875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="31.44140625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.33203125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.33203125" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.109375" style="1"/>
+    <col min="15" max="15" width="13.6640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="15.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="33.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="30.5546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="31.44140625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="27.33203125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="23.33203125" style="1" customWidth="1"/>
+    <col min="22" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:22" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2583,34 +2613,36 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="5"/>
-    </row>
-    <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B3" s="37" t="s">
+      <c r="T2" s="3"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="5"/>
+    </row>
+    <row r="3" spans="2:22" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B3" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="38"/>
-      <c r="P3" s="38"/>
-      <c r="Q3" s="38"/>
-      <c r="R3" s="38"/>
-      <c r="S3" s="38"/>
-      <c r="T3" s="39"/>
-      <c r="U3" s="5"/>
-    </row>
-    <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="50"/>
+      <c r="L3" s="50"/>
+      <c r="M3" s="50"/>
+      <c r="N3" s="50"/>
+      <c r="O3" s="50"/>
+      <c r="P3" s="50"/>
+      <c r="Q3" s="50"/>
+      <c r="R3" s="50"/>
+      <c r="S3" s="50"/>
+      <c r="T3" s="50"/>
+      <c r="U3" s="51"/>
+      <c r="V3" s="5"/>
+    </row>
+    <row r="4" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -2629,20 +2661,21 @@
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
       <c r="S4" s="7"/>
-      <c r="T4" s="8"/>
-    </row>
-    <row r="5" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="T4" s="7"/>
+      <c r="U4" s="8"/>
+    </row>
+    <row r="5" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6"/>
       <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="52"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
@@ -2652,20 +2685,21 @@
       <c r="Q5" s="17"/>
       <c r="R5" s="17"/>
       <c r="S5" s="17"/>
-      <c r="T5" s="18"/>
-    </row>
-    <row r="6" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="T5" s="17"/>
+      <c r="U5" s="18"/>
+    </row>
+    <row r="6" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6"/>
       <c r="C6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="53"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
@@ -2675,9 +2709,10 @@
       <c r="Q6" s="17"/>
       <c r="R6" s="17"/>
       <c r="S6" s="17"/>
-      <c r="T6" s="18"/>
-    </row>
-    <row r="7" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="T6" s="17"/>
+      <c r="U6" s="18"/>
+    </row>
+    <row r="7" spans="2:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6"/>
       <c r="C7" s="17"/>
       <c r="D7" s="19"/>
@@ -2696,9 +2731,10 @@
       <c r="Q7" s="17"/>
       <c r="R7" s="17"/>
       <c r="S7" s="17"/>
-      <c r="T7" s="18"/>
-    </row>
-    <row r="8" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="T7" s="17"/>
+      <c r="U7" s="18"/>
+    </row>
+    <row r="8" spans="2:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
@@ -2717,9 +2753,10 @@
       <c r="Q8" s="17"/>
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
-      <c r="T8" s="18"/>
-    </row>
-    <row r="9" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T8" s="17"/>
+      <c r="U8" s="18"/>
+    </row>
+    <row r="9" spans="2:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="15"/>
       <c r="C9" s="57" t="s">
         <v>1</v>
@@ -2736,25 +2773,26 @@
         <v>5</v>
       </c>
       <c r="K9" s="58" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L9" s="58"/>
       <c r="M9" s="58"/>
       <c r="N9" s="58"/>
       <c r="O9" s="58"/>
-      <c r="P9" s="57" t="s">
+      <c r="P9" s="58"/>
+      <c r="Q9" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="Q9" s="57"/>
       <c r="R9" s="57"/>
-      <c r="S9" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="T9" s="22" t="s">
+      <c r="S9" s="57"/>
+      <c r="T9" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="U9" s="22" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:22" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="16" t="s">
         <v>7</v>
       </c>
@@ -2774,10 +2812,10 @@
         <v>14</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J10" s="23" t="s">
         <v>15</v>
@@ -2795,47 +2833,50 @@
         <v>19</v>
       </c>
       <c r="O10" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="P10" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q10" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="P10" s="23" t="s">
+      <c r="R10" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="S10" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="Q10" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="R10" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="S10" s="24"/>
-      <c r="T10" s="25"/>
-    </row>
-    <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T10" s="24"/>
+      <c r="U10" s="25"/>
+    </row>
+    <row r="11" spans="2:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="9">
         <v>1</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="F11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="G11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="H11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="I11" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="J11" s="10" t="s">
         <v>33</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="J11" s="10" t="s">
-        <v>34</v>
       </c>
       <c r="K11" s="10">
         <v>0.24399999999999999</v>
@@ -2850,47 +2891,48 @@
         <v>0.216</v>
       </c>
       <c r="O11" s="10"/>
-      <c r="P11" s="10" t="s">
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="R11" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="Q11" s="10" t="s">
+      <c r="S11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="R11" s="10" t="s">
+      <c r="T11" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="S11" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="T11" s="11"/>
-    </row>
-    <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="U11" s="11"/>
+    </row>
+    <row r="12" spans="2:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>2</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="J12" s="10" t="s">
         <v>39</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I12" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="J12" s="10" t="s">
-        <v>40</v>
       </c>
       <c r="K12" s="10">
         <v>0.29299999999999998</v>
@@ -2905,43 +2947,44 @@
         <v>0.27400000000000002</v>
       </c>
       <c r="O12" s="10"/>
-      <c r="P12" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="R12" s="10"/>
-      <c r="S12" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="T12" s="11"/>
-    </row>
-    <row r="13" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S12" s="10"/>
+      <c r="T12" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="U12" s="11"/>
+    </row>
+    <row r="13" spans="2:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
         <v>3</v>
       </c>
       <c r="C13" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="J13" s="10" t="s">
         <v>41</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I13" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="J13" s="10" t="s">
-        <v>42</v>
       </c>
       <c r="K13" s="10">
         <v>0.252</v>
@@ -2956,47 +2999,48 @@
         <v>0.22</v>
       </c>
       <c r="O13" s="10"/>
-      <c r="P13" s="10" t="s">
+      <c r="P13" s="10"/>
+      <c r="Q13" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="R13" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="Q13" s="10" t="s">
+      <c r="S13" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="R13" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="S13" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="T13" s="11"/>
-    </row>
-    <row r="14" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T13" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="U13" s="11"/>
+    </row>
+    <row r="14" spans="2:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="9">
         <v>4</v>
       </c>
       <c r="C14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="E14" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="F14" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="G14" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="H14" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="I14" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="I14" s="10" t="s">
-        <v>47</v>
-      </c>
       <c r="J14" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K14" s="10">
         <v>0.248</v>
@@ -3015,33 +3059,34 @@
       <c r="Q14" s="10"/>
       <c r="R14" s="10"/>
       <c r="S14" s="10"/>
-      <c r="T14" s="11"/>
-    </row>
-    <row r="15" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T14" s="10"/>
+      <c r="U14" s="11"/>
+    </row>
+    <row r="15" spans="2:22" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="9">
         <v>5</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="G15" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="H15" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I15" s="10"/>
       <c r="J15" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K15" s="10">
         <v>0.28699999999999998</v>
@@ -3060,33 +3105,34 @@
       <c r="Q15" s="10"/>
       <c r="R15" s="10"/>
       <c r="S15" s="10"/>
-      <c r="T15" s="11"/>
-    </row>
-    <row r="16" spans="2:21" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T15" s="10"/>
+      <c r="U15" s="11"/>
+    </row>
+    <row r="16" spans="2:22" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="9">
         <v>6</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D16" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="G16" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="H16" s="26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I16" s="10"/>
       <c r="J16" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K16" s="10">
         <v>0.26</v>
@@ -3105,35 +3151,36 @@
       <c r="Q16" s="10"/>
       <c r="R16" s="10"/>
       <c r="S16" s="10"/>
-      <c r="T16" s="11"/>
-    </row>
-    <row r="17" spans="2:20" ht="95.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T16" s="10"/>
+      <c r="U16" s="11"/>
+    </row>
+    <row r="17" spans="2:21" ht="95.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="9">
         <v>7</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D17" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="G17" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H17" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J17" s="10" t="s">
         <v>66</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H17" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="I17" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="J17" s="10" t="s">
-        <v>67</v>
       </c>
       <c r="K17" s="10">
         <v>0.55300000000000005</v>
@@ -3148,43 +3195,44 @@
         <v>0.55300000000000005</v>
       </c>
       <c r="O17" s="10"/>
-      <c r="P17" s="10" t="s">
+      <c r="P17" s="10"/>
+      <c r="Q17" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="R17" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="Q17" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="R17" s="10"/>
       <c r="S17" s="10"/>
-      <c r="T17" s="11"/>
-    </row>
-    <row r="18" spans="2:20" ht="97.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T17" s="10"/>
+      <c r="U17" s="11"/>
+    </row>
+    <row r="18" spans="2:21" ht="97.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9">
         <v>8</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D18" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F18" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="10" t="s">
+      <c r="G18" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H18" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="G18" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H18" s="26" t="s">
+      <c r="I18" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J18" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K18" s="10">
         <v>0.59599999999999997</v>
@@ -3199,43 +3247,44 @@
         <v>0.59699999999999998</v>
       </c>
       <c r="O18" s="10"/>
-      <c r="P18" s="10" t="s">
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="R18" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="Q18" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="R18" s="10"/>
       <c r="S18" s="10"/>
-      <c r="T18" s="11"/>
-    </row>
-    <row r="19" spans="2:20" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T18" s="10"/>
+      <c r="U18" s="11"/>
+    </row>
+    <row r="19" spans="2:21" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>9</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D19" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F19" s="10" t="s">
+      <c r="G19" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="G19" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H19" s="26" t="s">
+      <c r="I19" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="I19" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J19" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K19" s="10">
         <v>0.71</v>
@@ -3250,43 +3299,44 @@
         <v>0.71299999999999997</v>
       </c>
       <c r="O19" s="10"/>
-      <c r="P19" s="10" t="s">
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="R19" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="Q19" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="R19" s="10"/>
       <c r="S19" s="10"/>
-      <c r="T19" s="11"/>
-    </row>
-    <row r="20" spans="2:20" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T19" s="10"/>
+      <c r="U19" s="11"/>
+    </row>
+    <row r="20" spans="2:21" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="9">
         <v>10</v>
       </c>
       <c r="C20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="F20" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F20" s="10" t="s">
+      <c r="G20" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H20" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="G20" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H20" s="26" t="s">
+      <c r="I20" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="I20" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J20" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K20" s="10">
         <v>0.76400000000000001</v>
@@ -3301,43 +3351,44 @@
         <v>0.76700000000000002</v>
       </c>
       <c r="O20" s="10"/>
-      <c r="P20" s="10" t="s">
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="R20" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="Q20" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="R20" s="10"/>
       <c r="S20" s="10"/>
-      <c r="T20" s="11"/>
-    </row>
-    <row r="21" spans="2:20" ht="81" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T20" s="10"/>
+      <c r="U20" s="11"/>
+    </row>
+    <row r="21" spans="2:21" ht="81" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9">
         <v>11</v>
       </c>
       <c r="C21" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H21" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F21" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H21" s="26" t="s">
+      <c r="I21" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J21" s="10" t="s">
         <v>72</v>
-      </c>
-      <c r="I21" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="J21" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="K21" s="10">
         <v>0.79100000000000004</v>
@@ -3352,45 +3403,46 @@
         <v>0.79300000000000004</v>
       </c>
       <c r="O21" s="10"/>
-      <c r="P21" s="10" t="s">
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="R21" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="Q21" s="10" t="s">
+      <c r="S21" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="R21" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="S21" s="10"/>
-      <c r="T21" s="11"/>
-    </row>
-    <row r="22" spans="2:20" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T21" s="10"/>
+      <c r="U21" s="11"/>
+    </row>
+    <row r="22" spans="2:21" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
         <v>12</v>
       </c>
       <c r="C22" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H22" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="D22" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H22" s="26" t="s">
-        <v>75</v>
-      </c>
       <c r="I22" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J22" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K22" s="10">
         <v>0.79600000000000004</v>
@@ -3405,61 +3457,116 @@
         <v>0.79900000000000004</v>
       </c>
       <c r="O22" s="10"/>
-      <c r="P22" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q22" s="10"/>
-      <c r="R22" s="10"/>
-      <c r="S22" s="10"/>
-      <c r="T22" s="11"/>
-    </row>
-    <row r="23" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P22" s="10"/>
+      <c r="Q22" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="R22" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="S22" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="T22" s="10"/>
+      <c r="U22" s="11"/>
+    </row>
+    <row r="23" spans="2:21" ht="94.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
+      <c r="C23" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J23" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="K23" s="10">
+        <v>0.88900000000000001</v>
+      </c>
+      <c r="L23" s="10">
+        <v>0.89100000000000001</v>
+      </c>
+      <c r="M23" s="10">
+        <v>0.88900000000000001</v>
+      </c>
+      <c r="N23" s="10">
+        <v>0.88900000000000001</v>
+      </c>
       <c r="O23" s="10"/>
       <c r="P23" s="10"/>
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
       <c r="S23" s="10"/>
-      <c r="T23" s="11"/>
-    </row>
-    <row r="24" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T23" s="10"/>
+      <c r="U23" s="11"/>
+    </row>
+    <row r="24" spans="2:21" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9">
         <v>14</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
+      <c r="C24" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J24" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="K24" s="10">
+        <v>0.89500000000000002</v>
+      </c>
+      <c r="L24" s="10">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="M24" s="10">
+        <v>0.89500000000000002</v>
+      </c>
+      <c r="N24" s="10">
+        <v>0.89500000000000002</v>
+      </c>
       <c r="O24" s="10"/>
       <c r="P24" s="10"/>
       <c r="Q24" s="10"/>
       <c r="R24" s="10"/>
       <c r="S24" s="10"/>
-      <c r="T24" s="11"/>
-    </row>
-    <row r="25" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T24" s="10"/>
+      <c r="U24" s="11"/>
+    </row>
+    <row r="25" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9">
         <v>15</v>
       </c>
@@ -3480,9 +3587,10 @@
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="10"/>
-      <c r="T25" s="11"/>
-    </row>
-    <row r="26" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T25" s="10"/>
+      <c r="U25" s="11"/>
+    </row>
+    <row r="26" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
         <v>16</v>
       </c>
@@ -3503,9 +3611,10 @@
       <c r="Q26" s="10"/>
       <c r="R26" s="10"/>
       <c r="S26" s="10"/>
-      <c r="T26" s="11"/>
-    </row>
-    <row r="27" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T26" s="10"/>
+      <c r="U26" s="11"/>
+    </row>
+    <row r="27" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="9">
         <v>17</v>
       </c>
@@ -3526,9 +3635,10 @@
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
       <c r="S27" s="10"/>
-      <c r="T27" s="11"/>
-    </row>
-    <row r="28" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T27" s="10"/>
+      <c r="U27" s="11"/>
+    </row>
+    <row r="28" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="9">
         <v>18</v>
       </c>
@@ -3549,9 +3659,10 @@
       <c r="Q28" s="10"/>
       <c r="R28" s="10"/>
       <c r="S28" s="10"/>
-      <c r="T28" s="11"/>
-    </row>
-    <row r="29" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T28" s="10"/>
+      <c r="U28" s="11"/>
+    </row>
+    <row r="29" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="9">
         <v>19</v>
       </c>
@@ -3572,9 +3683,10 @@
       <c r="Q29" s="10"/>
       <c r="R29" s="10"/>
       <c r="S29" s="10"/>
-      <c r="T29" s="11"/>
-    </row>
-    <row r="30" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T29" s="10"/>
+      <c r="U29" s="11"/>
+    </row>
+    <row r="30" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="9">
         <v>20</v>
       </c>
@@ -3595,9 +3707,10 @@
       <c r="Q30" s="10"/>
       <c r="R30" s="10"/>
       <c r="S30" s="10"/>
-      <c r="T30" s="11"/>
-    </row>
-    <row r="31" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T30" s="10"/>
+      <c r="U30" s="11"/>
+    </row>
+    <row r="31" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="9">
         <v>21</v>
       </c>
@@ -3618,9 +3731,10 @@
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
       <c r="S31" s="10"/>
-      <c r="T31" s="11"/>
-    </row>
-    <row r="32" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T31" s="10"/>
+      <c r="U31" s="11"/>
+    </row>
+    <row r="32" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9">
         <v>22</v>
       </c>
@@ -3641,9 +3755,10 @@
       <c r="Q32" s="10"/>
       <c r="R32" s="10"/>
       <c r="S32" s="10"/>
-      <c r="T32" s="11"/>
-    </row>
-    <row r="33" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T32" s="10"/>
+      <c r="U32" s="11"/>
+    </row>
+    <row r="33" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="9">
         <v>23</v>
       </c>
@@ -3664,9 +3779,10 @@
       <c r="Q33" s="10"/>
       <c r="R33" s="10"/>
       <c r="S33" s="10"/>
-      <c r="T33" s="11"/>
-    </row>
-    <row r="34" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T33" s="10"/>
+      <c r="U33" s="11"/>
+    </row>
+    <row r="34" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="9">
         <v>24</v>
       </c>
@@ -3687,9 +3803,10 @@
       <c r="Q34" s="10"/>
       <c r="R34" s="10"/>
       <c r="S34" s="10"/>
-      <c r="T34" s="11"/>
-    </row>
-    <row r="35" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T34" s="10"/>
+      <c r="U34" s="11"/>
+    </row>
+    <row r="35" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="9">
         <v>25</v>
       </c>
@@ -3710,9 +3827,10 @@
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
       <c r="S35" s="10"/>
-      <c r="T35" s="11"/>
-    </row>
-    <row r="36" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T35" s="10"/>
+      <c r="U35" s="11"/>
+    </row>
+    <row r="36" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9">
         <v>26</v>
       </c>
@@ -3733,9 +3851,10 @@
       <c r="Q36" s="10"/>
       <c r="R36" s="10"/>
       <c r="S36" s="10"/>
-      <c r="T36" s="11"/>
-    </row>
-    <row r="37" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T36" s="10"/>
+      <c r="U36" s="11"/>
+    </row>
+    <row r="37" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="9">
         <v>27</v>
       </c>
@@ -3756,9 +3875,10 @@
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
       <c r="S37" s="10"/>
-      <c r="T37" s="11"/>
-    </row>
-    <row r="38" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T37" s="10"/>
+      <c r="U37" s="11"/>
+    </row>
+    <row r="38" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="9">
         <v>28</v>
       </c>
@@ -3779,9 +3899,10 @@
       <c r="Q38" s="10"/>
       <c r="R38" s="10"/>
       <c r="S38" s="10"/>
-      <c r="T38" s="11"/>
-    </row>
-    <row r="39" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T38" s="10"/>
+      <c r="U38" s="11"/>
+    </row>
+    <row r="39" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
         <v>29</v>
       </c>
@@ -3802,9 +3923,10 @@
       <c r="Q39" s="10"/>
       <c r="R39" s="10"/>
       <c r="S39" s="10"/>
-      <c r="T39" s="11"/>
-    </row>
-    <row r="40" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T39" s="10"/>
+      <c r="U39" s="11"/>
+    </row>
+    <row r="40" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9">
         <v>30</v>
       </c>
@@ -3825,9 +3947,10 @@
       <c r="Q40" s="10"/>
       <c r="R40" s="10"/>
       <c r="S40" s="10"/>
-      <c r="T40" s="11"/>
-    </row>
-    <row r="41" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T40" s="10"/>
+      <c r="U40" s="11"/>
+    </row>
+    <row r="41" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="9">
         <v>31</v>
       </c>
@@ -3848,9 +3971,10 @@
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
       <c r="S41" s="10"/>
-      <c r="T41" s="11"/>
-    </row>
-    <row r="42" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T41" s="10"/>
+      <c r="U41" s="11"/>
+    </row>
+    <row r="42" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="9">
         <v>32</v>
       </c>
@@ -3871,9 +3995,10 @@
       <c r="Q42" s="10"/>
       <c r="R42" s="10"/>
       <c r="S42" s="10"/>
-      <c r="T42" s="11"/>
-    </row>
-    <row r="43" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T42" s="10"/>
+      <c r="U42" s="11"/>
+    </row>
+    <row r="43" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="9">
         <v>33</v>
       </c>
@@ -3894,9 +4019,10 @@
       <c r="Q43" s="10"/>
       <c r="R43" s="10"/>
       <c r="S43" s="10"/>
-      <c r="T43" s="11"/>
-    </row>
-    <row r="44" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T43" s="10"/>
+      <c r="U43" s="11"/>
+    </row>
+    <row r="44" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="9">
         <v>34</v>
       </c>
@@ -3917,9 +4043,10 @@
       <c r="Q44" s="10"/>
       <c r="R44" s="10"/>
       <c r="S44" s="10"/>
-      <c r="T44" s="11"/>
-    </row>
-    <row r="45" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T44" s="10"/>
+      <c r="U44" s="11"/>
+    </row>
+    <row r="45" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="9">
         <v>35</v>
       </c>
@@ -3940,9 +4067,10 @@
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
       <c r="S45" s="10"/>
-      <c r="T45" s="11"/>
-    </row>
-    <row r="46" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T45" s="10"/>
+      <c r="U45" s="11"/>
+    </row>
+    <row r="46" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="9">
         <v>36</v>
       </c>
@@ -3963,9 +4091,10 @@
       <c r="Q46" s="10"/>
       <c r="R46" s="10"/>
       <c r="S46" s="10"/>
-      <c r="T46" s="11"/>
-    </row>
-    <row r="47" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T46" s="10"/>
+      <c r="U46" s="11"/>
+    </row>
+    <row r="47" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="9">
         <v>37</v>
       </c>
@@ -3986,9 +4115,10 @@
       <c r="Q47" s="10"/>
       <c r="R47" s="10"/>
       <c r="S47" s="10"/>
-      <c r="T47" s="11"/>
-    </row>
-    <row r="48" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T47" s="10"/>
+      <c r="U47" s="11"/>
+    </row>
+    <row r="48" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="9">
         <v>38</v>
       </c>
@@ -4009,9 +4139,10 @@
       <c r="Q48" s="10"/>
       <c r="R48" s="10"/>
       <c r="S48" s="10"/>
-      <c r="T48" s="11"/>
-    </row>
-    <row r="49" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T48" s="10"/>
+      <c r="U48" s="11"/>
+    </row>
+    <row r="49" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="9">
         <v>39</v>
       </c>
@@ -4032,9 +4163,10 @@
       <c r="Q49" s="10"/>
       <c r="R49" s="10"/>
       <c r="S49" s="10"/>
-      <c r="T49" s="11"/>
-    </row>
-    <row r="50" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T49" s="10"/>
+      <c r="U49" s="11"/>
+    </row>
+    <row r="50" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="9">
         <v>40</v>
       </c>
@@ -4055,9 +4187,10 @@
       <c r="Q50" s="10"/>
       <c r="R50" s="10"/>
       <c r="S50" s="10"/>
-      <c r="T50" s="11"/>
-    </row>
-    <row r="51" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T50" s="10"/>
+      <c r="U50" s="11"/>
+    </row>
+    <row r="51" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="9">
         <v>41</v>
       </c>
@@ -4078,22 +4211,23 @@
       <c r="Q51" s="12"/>
       <c r="R51" s="12"/>
       <c r="S51" s="12"/>
-      <c r="T51" s="13"/>
-    </row>
-    <row r="52" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T51" s="12"/>
+      <c r="U51" s="13"/>
+    </row>
+    <row r="52" spans="2:21" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C52" s="14" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="B3:U3"/>
     <mergeCell ref="D5:J5"/>
     <mergeCell ref="D6:J6"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="E9:I9"/>
-    <mergeCell ref="K9:O9"/>
-    <mergeCell ref="P9:R9"/>
+    <mergeCell ref="K9:P9"/>
+    <mergeCell ref="Q9:S9"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add notes for distilbert model
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\git-school\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42CAFEE-C635-4AD6-AD2D-5AAD5CBE8437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0787EF69-4B7D-4310-9CA1-308EBAED11DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="100">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -348,6 +348,12 @@
   </si>
   <si>
     <t>BERT-base-uncased</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We started off using a DistilBERT model, which is a lightweight version of the base BERT model. The specific model we ended up using was the "DistilBERT-base-uncased-sst-2-english" model, which is a finetuned model for emotion classification for English. The model was already trained on a large corpus of data, so we only had to change the classification head to match our desired output (6 classes + neutral) and finetune the model for a small number of layers until a satisfactory performance is reached. When evaluated on the validation set, the model showed a promising performance, outperforming the best model we had previously, the LSTM-v3 architecture. The weighted F1 score and the accuracy were both 88.9%. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The first downside of this model is that it takes a considerable amount of time to fine-tune. We only trained the model for a small number of epochs, between 3 and 5, and that took between 20 and 30 minutes for each run. The second downside is that it greatly overfits the training data. When evaluated on the validation set, which consists of a held-out percentage of the dataset used for finetuning, it achieves an incredible performance of about 89%. However, when we used our test set, the show dataset, the performance plummeted to 51% for accuracy and 44% for the weighted F1 score. This shows that the current approach causes the model to learn the hidden intrinsic patterns of the dataset used for training and perform very well when evaluated on a subset of it. However, when the test set is a new, never-seen dataset, the performance plummets as the model fails to generalize across multiple datasets well. </t>
   </si>
 </sst>
 </file>
@@ -771,64 +777,64 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1219,27 +1225,27 @@
       <c r="U2" s="5"/>
     </row>
     <row r="3" spans="2:21" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="51"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="38"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="39"/>
       <c r="U3" s="5"/>
     </row>
     <row r="4" spans="2:21" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -1268,13 +1274,13 @@
       <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
@@ -1291,13 +1297,13 @@
       <c r="C6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
@@ -1395,26 +1401,26 @@
     </row>
     <row r="11" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="27"/>
-      <c r="C11" s="54" t="s">
+      <c r="C11" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="55"/>
-      <c r="E11" s="55"/>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="55"/>
-      <c r="J11" s="55"/>
-      <c r="K11" s="55"/>
-      <c r="L11" s="55"/>
-      <c r="M11" s="55"/>
-      <c r="N11" s="55"/>
-      <c r="O11" s="55"/>
-      <c r="P11" s="55"/>
-      <c r="Q11" s="55"/>
-      <c r="R11" s="55"/>
-      <c r="S11" s="55"/>
-      <c r="T11" s="55"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
+      <c r="Q11" s="43"/>
+      <c r="R11" s="43"/>
+      <c r="S11" s="43"/>
+      <c r="T11" s="43"/>
     </row>
     <row r="12" spans="2:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="27"/>
@@ -1443,13 +1449,13 @@
       <c r="D13" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="56"/>
-      <c r="F13" s="56"/>
-      <c r="G13" s="56"/>
-      <c r="H13" s="56"/>
-      <c r="I13" s="56"/>
-      <c r="J13" s="56"/>
-      <c r="K13" s="56"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
       <c r="L13" s="32"/>
       <c r="M13" s="32"/>
       <c r="N13" s="32"/>
@@ -1466,13 +1472,13 @@
       <c r="D14" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="47"/>
-      <c r="J14" s="47"/>
-      <c r="K14" s="47"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="45"/>
       <c r="L14" s="32"/>
       <c r="M14" s="32"/>
       <c r="N14" s="32"/>
@@ -1526,79 +1532,79 @@
       <c r="T16" s="32"/>
     </row>
     <row r="17" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="44"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="41" t="s">
+      <c r="B17" s="46"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="41"/>
-      <c r="F17" s="39" t="s">
+      <c r="E17" s="49"/>
+      <c r="F17" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="41" t="s">
+      <c r="G17" s="51"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="L17" s="39" t="s">
+      <c r="L17" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="M17" s="39"/>
-      <c r="N17" s="39"/>
-      <c r="O17" s="39"/>
-      <c r="P17" s="39"/>
-      <c r="Q17" s="41" t="s">
+      <c r="M17" s="51"/>
+      <c r="N17" s="51"/>
+      <c r="O17" s="51"/>
+      <c r="P17" s="51"/>
+      <c r="Q17" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="R17" s="41"/>
-      <c r="S17" s="41"/>
-      <c r="T17" s="39" t="s">
+      <c r="R17" s="49"/>
+      <c r="S17" s="49"/>
+      <c r="T17" s="51" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="44"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="38"/>
-      <c r="L18" s="40" t="s">
+      <c r="B18" s="46"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="52"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="52"/>
+      <c r="I18" s="52"/>
+      <c r="J18" s="52"/>
+      <c r="K18" s="50"/>
+      <c r="L18" s="56" t="s">
         <v>55</v>
       </c>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
-      <c r="O18" s="40"/>
-      <c r="P18" s="40"/>
-      <c r="Q18" s="38"/>
-      <c r="R18" s="38"/>
-      <c r="S18" s="38"/>
-      <c r="T18" s="42"/>
+      <c r="M18" s="56"/>
+      <c r="N18" s="56"/>
+      <c r="O18" s="56"/>
+      <c r="P18" s="56"/>
+      <c r="Q18" s="50"/>
+      <c r="R18" s="50"/>
+      <c r="S18" s="50"/>
+      <c r="T18" s="52"/>
     </row>
     <row r="19" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="44"/>
-      <c r="C19" s="45" t="s">
+      <c r="B19" s="46"/>
+      <c r="C19" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="37" t="s">
+      <c r="E19" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="F19" s="43" t="s">
+      <c r="F19" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="G19" s="43" t="s">
+      <c r="G19" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="43" t="s">
+      <c r="H19" s="53" t="s">
         <v>14</v>
       </c>
       <c r="I19" s="33" t="s">
@@ -1607,61 +1613,61 @@
       <c r="J19" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="K19" s="37" t="s">
+      <c r="K19" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="L19" s="43" t="s">
+      <c r="L19" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="M19" s="43" t="s">
+      <c r="M19" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="N19" s="43" t="s">
+      <c r="N19" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="O19" s="43" t="s">
+      <c r="O19" s="53" t="s">
         <v>19</v>
       </c>
       <c r="P19" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="Q19" s="37" t="s">
+      <c r="Q19" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="R19" s="37" t="s">
+      <c r="R19" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="S19" s="37" t="s">
+      <c r="S19" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="T19" s="43"/>
+      <c r="T19" s="53"/>
     </row>
     <row r="20" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="44"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
       <c r="I20" s="34" t="s">
         <v>57</v>
       </c>
       <c r="J20" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="K20" s="38"/>
-      <c r="L20" s="42"/>
-      <c r="M20" s="42"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="42"/>
+      <c r="K20" s="50"/>
+      <c r="L20" s="52"/>
+      <c r="M20" s="52"/>
+      <c r="N20" s="52"/>
+      <c r="O20" s="52"/>
       <c r="P20" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="Q20" s="38"/>
-      <c r="R20" s="38"/>
-      <c r="S20" s="38"/>
-      <c r="T20" s="42"/>
+      <c r="Q20" s="50"/>
+      <c r="R20" s="50"/>
+      <c r="S20" s="50"/>
+      <c r="T20" s="52"/>
     </row>
     <row r="21" spans="2:20" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="27"/>
@@ -2530,27 +2536,6 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B3:T3"/>
-    <mergeCell ref="D5:J5"/>
-    <mergeCell ref="D6:J6"/>
-    <mergeCell ref="C11:T11"/>
-    <mergeCell ref="E13:K13"/>
-    <mergeCell ref="E14:K14"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:E18"/>
-    <mergeCell ref="F17:J18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
     <mergeCell ref="S19:S20"/>
     <mergeCell ref="L17:P17"/>
     <mergeCell ref="L18:P18"/>
@@ -2561,6 +2546,27 @@
     <mergeCell ref="O19:O20"/>
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="E14:K14"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:E18"/>
+    <mergeCell ref="F17:J18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="C11:T11"/>
+    <mergeCell ref="E13:K13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2618,28 +2624,28 @@
       <c r="V2" s="5"/>
     </row>
     <row r="3" spans="2:22" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="50"/>
-      <c r="U3" s="51"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="38"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="38"/>
+      <c r="U3" s="39"/>
       <c r="V3" s="5"/>
     </row>
     <row r="4" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.45">
@@ -2669,13 +2675,13 @@
       <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
@@ -2693,13 +2699,13 @@
       <c r="C6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
@@ -3470,7 +3476,7 @@
       <c r="T22" s="10"/>
       <c r="U22" s="11"/>
     </row>
-    <row r="23" spans="2:21" ht="94.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:21" ht="405.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
@@ -3510,10 +3516,18 @@
       <c r="N23" s="10">
         <v>0.88900000000000001</v>
       </c>
-      <c r="O23" s="10"/>
-      <c r="P23" s="10"/>
-      <c r="Q23" s="10"/>
-      <c r="R23" s="10"/>
+      <c r="O23" s="10">
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="P23" s="10">
+        <v>0.438</v>
+      </c>
+      <c r="Q23" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="R23" s="10" t="s">
+        <v>99</v>
+      </c>
       <c r="S23" s="10"/>
       <c r="T23" s="10"/>
       <c r="U23" s="11"/>
@@ -3558,8 +3572,12 @@
       <c r="N24" s="10">
         <v>0.89500000000000002</v>
       </c>
-      <c r="O24" s="10"/>
-      <c r="P24" s="10"/>
+      <c r="O24" s="10">
+        <v>0.48099999999999998</v>
+      </c>
+      <c r="P24" s="10">
+        <v>0.38200000000000001</v>
+      </c>
       <c r="Q24" s="10"/>
       <c r="R24" s="10"/>
       <c r="S24" s="10"/>

</xml_diff>

<commit_message>
Updat model iteration xlsx file
</commit_message>
<xml_diff>
--- a/deliverables/Task 6/Y2A_model_iteration_log.xlsx
+++ b/deliverables/Task 6/Y2A_model_iteration_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rzvn1\Documents\git-school\fae2-nlpr-group-group-12-1\deliverables\Task 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0787EF69-4B7D-4310-9CA1-308EBAED11DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E2A73F-6405-4470-B74F-381127ACE26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6D8ECC7B-96E6-4221-81CD-57BD062A831A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="102">
   <si>
     <t>Model iteration log</t>
   </si>
@@ -354,6 +354,12 @@
   </si>
   <si>
     <t xml:space="preserve">The first downside of this model is that it takes a considerable amount of time to fine-tune. We only trained the model for a small number of epochs, between 3 and 5, and that took between 20 and 30 minutes for each run. The second downside is that it greatly overfits the training data. When evaluated on the validation set, which consists of a held-out percentage of the dataset used for finetuning, it achieves an incredible performance of about 89%. However, when we used our test set, the show dataset, the performance plummeted to 51% for accuracy and 44% for the weighted F1 score. This shows that the current approach causes the model to learn the hidden intrinsic patterns of the dataset used for training and perform very well when evaluated on a subset of it. However, when the test set is a new, never-seen dataset, the performance plummets as the model fails to generalize across multiple datasets well. </t>
+  </si>
+  <si>
+    <t>The second model we tried was the bert-base-uncased model. We tried this model as it has more parameters than the DistilBERT model we previously tried, and we believed that the increased number of parameters it has would help it better understand and create meaningful representations of the training data. We again changed the classification head to match our desired output (6 classes + neutral) and then we finetuned the model for a small number of epochs until a satisfactory performance was reached. We then used the held out evaluation set to test the performance of this new model and results were indeede better than the ones achieved by the DistilBERT model and much better than anything previously achieved. The model achieved an accuracy and weighted F1 score of 89.5%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The model took a significant amount of time to fine-tune. We only trained it for 5 epochs, and the training process took around 40-45 minutes to complete. Another major issue with this model is that its performance doesn’t extend across multiple datasets. When evaluated on the validation set, it achieved an excellent performance of nearly 90%. However, when we tested the model's performance on the show data, annotated by the company's pipeline, the results were far from our expectations. Although this model performed better during training and on the validation set compared to the previously evaluated DistilBERT model, it performed even worse on the test data. Its accuracy dropped to 48.1%, and the weighted F1 score decreased further, reaching 38.2%. This indicates that both models, despite performing well on the evaluation set, did not truly learn relevant linguistic patterns or significant, emotion-filled words during training and were only overfitting to that specific dataset. When tested on a different dataset, their true capabilities became evident. </t>
   </si>
 </sst>
 </file>
@@ -3476,7 +3482,7 @@
       <c r="T22" s="10"/>
       <c r="U22" s="11"/>
     </row>
-    <row r="23" spans="2:21" ht="405.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:21" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
         <v>13</v>
       </c>
@@ -3532,7 +3538,7 @@
       <c r="T23" s="10"/>
       <c r="U23" s="11"/>
     </row>
-    <row r="24" spans="2:21" ht="90.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:21" ht="396" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9">
         <v>14</v>
       </c>
@@ -3578,8 +3584,12 @@
       <c r="P24" s="10">
         <v>0.38200000000000001</v>
       </c>
-      <c r="Q24" s="10"/>
-      <c r="R24" s="10"/>
+      <c r="Q24" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="R24" s="10" t="s">
+        <v>101</v>
+      </c>
       <c r="S24" s="10"/>
       <c r="T24" s="10"/>
       <c r="U24" s="11"/>

</xml_diff>